<commit_message>
Update thickness standards: add tolerance_mm column, update sync script and UI
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -5,19 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tam.nguyen\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
   <sheets>
     <sheet name="Tháng 04.2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
-    <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
     <definedName name="\0">#REF!</definedName>
@@ -1347,9 +1346,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="[$-1000000]00000"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="[$-1000000]00000"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -1561,7 +1560,7 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1618,16 +1617,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1652,7 +1651,7 @@
     <xf numFmtId="2" fontId="7" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1670,16 +1669,16 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="3" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4008,60 +4007,6 @@
         </row>
       </sheetData>
       <sheetData sheetId="5"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Detail in Aug"/>
-      <sheetName val="247"/>
-      <sheetName val="BCC"/>
-      <sheetName val="Sheet3"/>
-      <sheetName val="Sheet1"/>
-      <sheetName val="OT 6 tháng"/>
-      <sheetName val="Sản Lượng Ngày"/>
-      <sheetName val="VỆ SINH T4.2026"/>
-      <sheetName val="Tháng 04.2026"/>
-      <sheetName val="Activities T4"/>
-      <sheetName val="Tổng hợp tuần T02"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="cập nhật mới không tính PPH T1"/>
-      <sheetName val="T12"/>
-      <sheetName val="ds đi hổ trợ"/>
-      <sheetName val="Đổ"/>
-      <sheetName val="FOAMING_POURING"/>
-      <sheetName val="Tách"/>
-      <sheetName val="FOAMING_SPLITTING"/>
-      <sheetName val="Sheet5"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -4367,20 +4312,20 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:BC142"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K142"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="27.6640625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5703125" style="43" customWidth="1"/>
-    <col min="8" max="8" width="27.5703125" style="43" customWidth="1"/>
-    <col min="9" max="9" width="19.5703125" style="43" customWidth="1"/>
-    <col min="10" max="10" width="18.42578125" customWidth="1"/>
-    <col min="11" max="11" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" style="43" customWidth="1"/>
+    <col min="8" max="8" width="27.5546875" style="43" customWidth="1"/>
+    <col min="9" max="9" width="19.5546875" style="43" customWidth="1"/>
+    <col min="10" max="10" width="18.44140625" customWidth="1"/>
+    <col min="11" max="11" width="31.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:9" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -4390,14 +4335,14 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="3:9" s="1" customFormat="1" ht="19.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:9" s="1" customFormat="1" ht="18.600000000000001" x14ac:dyDescent="0.3">
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="4"/>
       <c r="H2" s="3"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C3" s="5" t="s">
         <v>0</v>
       </c>
@@ -4409,7 +4354,7 @@
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
     </row>
-    <row r="4" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C4" s="5" t="s">
         <v>2</v>
       </c>
@@ -4421,7 +4366,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
@@ -4433,7 +4378,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
@@ -4445,7 +4390,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
@@ -4457,7 +4402,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="5" t="s">
         <v>10</v>
       </c>
@@ -4469,7 +4414,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -4481,7 +4426,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -4493,7 +4438,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="11" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C11" s="5" t="s">
         <v>16</v>
       </c>
@@ -4505,7 +4450,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C12" s="5" t="s">
         <v>18</v>
       </c>
@@ -4517,7 +4462,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="13" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C13" s="5" t="s">
         <v>20</v>
       </c>
@@ -4529,7 +4474,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="14" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C14" s="5" t="s">
         <v>22</v>
       </c>
@@ -4541,7 +4486,7 @@
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
     </row>
-    <row r="15" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="5" t="s">
         <v>24</v>
       </c>
@@ -4553,7 +4498,7 @@
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:9" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C16" s="5" t="s">
         <v>26</v>
       </c>
@@ -4565,7 +4510,7 @@
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="1:11" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" s="7" customFormat="1" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="5" t="s">
         <v>28</v>
       </c>
@@ -4577,7 +4522,7 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="1:11" s="7" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" s="7" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="5" t="s">
         <v>30</v>
       </c>
@@ -4592,14 +4537,14 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" s="13" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" s="13" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F19" s="14"/>
       <c r="G19" s="15"/>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="17"/>
     </row>
-    <row r="20" spans="1:11" s="19" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" s="19" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
       <c r="E20" s="20"/>
@@ -4644,7 +4589,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4679,7 +4624,7 @@
       </c>
       <c r="K22" s="44"/>
     </row>
-    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4714,7 +4659,7 @@
       </c>
       <c r="K23" s="44"/>
     </row>
-    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4749,7 +4694,7 @@
       </c>
       <c r="K24" s="44"/>
     </row>
-    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4784,7 +4729,7 @@
       </c>
       <c r="K25" s="44"/>
     </row>
-    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="18" t="s">
         <v>56</v>
       </c>
@@ -4819,7 +4764,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4853,7 +4798,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="s">
         <v>63</v>
       </c>
@@ -4888,7 +4833,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="18" t="s">
         <v>65</v>
       </c>
@@ -4923,7 +4868,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="18" t="s">
         <v>67</v>
       </c>
@@ -4958,7 +4903,7 @@
       </c>
       <c r="K30" s="45"/>
     </row>
-    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4993,7 +4938,7 @@
       </c>
       <c r="K31" s="45"/>
     </row>
-    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5028,7 +4973,7 @@
       </c>
       <c r="K32" s="45"/>
     </row>
-    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5063,7 +5008,7 @@
       </c>
       <c r="K33" s="45"/>
     </row>
-    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5098,7 +5043,7 @@
       </c>
       <c r="K34" s="45"/>
     </row>
-    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5133,7 +5078,7 @@
       </c>
       <c r="K35" s="45"/>
     </row>
-    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5168,7 +5113,7 @@
       </c>
       <c r="K36" s="45"/>
     </row>
-    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5203,7 +5148,7 @@
       </c>
       <c r="K37" s="45"/>
     </row>
-    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5238,7 +5183,7 @@
       </c>
       <c r="K38" s="45"/>
     </row>
-    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5273,7 +5218,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5308,7 +5253,7 @@
       </c>
       <c r="K40" s="45"/>
     </row>
-    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5343,7 +5288,7 @@
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5378,7 +5323,7 @@
       </c>
       <c r="K42" s="45"/>
     </row>
-    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5413,7 +5358,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5448,7 +5393,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5483,7 +5428,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
         <v>105</v>
       </c>
@@ -5518,7 +5463,7 @@
       </c>
       <c r="K46" s="45"/>
     </row>
-    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5553,7 +5498,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5588,7 +5533,7 @@
       </c>
       <c r="K48" s="45"/>
     </row>
-    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="18" t="s">
         <v>111</v>
       </c>
@@ -5623,7 +5568,7 @@
       </c>
       <c r="K49" s="45"/>
     </row>
-    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5658,7 +5603,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5693,7 +5638,7 @@
       </c>
       <c r="K51" s="45"/>
     </row>
-    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5728,7 +5673,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="s">
         <v>119</v>
       </c>
@@ -5763,7 +5708,7 @@
       </c>
       <c r="K53" s="45"/>
     </row>
-    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5798,7 +5743,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5833,7 +5778,7 @@
       </c>
       <c r="K55" s="45"/>
     </row>
-    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5868,7 +5813,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5903,7 +5848,7 @@
       </c>
       <c r="K57" s="45"/>
     </row>
-    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5938,7 +5883,7 @@
       </c>
       <c r="K58" s="45"/>
     </row>
-    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5973,7 +5918,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6008,7 +5953,7 @@
       </c>
       <c r="K60" s="45"/>
     </row>
-    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6043,7 +5988,7 @@
       </c>
       <c r="K61" s="45"/>
     </row>
-    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="18" t="s">
         <v>138</v>
       </c>
@@ -6078,7 +6023,7 @@
       </c>
       <c r="K62" s="45"/>
     </row>
-    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6113,7 +6058,7 @@
       </c>
       <c r="K63" s="45"/>
     </row>
-    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6148,7 +6093,7 @@
       </c>
       <c r="K64" s="45"/>
     </row>
-    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="18" t="s">
         <v>145</v>
       </c>
@@ -6183,7 +6128,7 @@
       </c>
       <c r="K65" s="45"/>
     </row>
-    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6218,7 +6163,7 @@
       </c>
       <c r="K66" s="45"/>
     </row>
-    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6253,7 +6198,7 @@
       </c>
       <c r="K67" s="45"/>
     </row>
-    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="18" t="s">
         <v>151</v>
       </c>
@@ -6288,7 +6233,7 @@
       </c>
       <c r="K68" s="45"/>
     </row>
-    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6323,7 +6268,7 @@
       </c>
       <c r="K69" s="45"/>
     </row>
-    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6358,7 +6303,7 @@
       </c>
       <c r="K70" s="45"/>
     </row>
-    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="18" t="s">
         <v>157</v>
       </c>
@@ -6393,7 +6338,7 @@
       </c>
       <c r="K71" s="45"/>
     </row>
-    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6428,7 +6373,7 @@
       </c>
       <c r="K72" s="45"/>
     </row>
-    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6463,7 +6408,7 @@
       </c>
       <c r="K73" s="45"/>
     </row>
-    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="18" t="s">
         <v>163</v>
       </c>
@@ -6498,7 +6443,7 @@
       </c>
       <c r="K74" s="45"/>
     </row>
-    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6533,7 +6478,7 @@
       </c>
       <c r="K75" s="45"/>
     </row>
-    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="18" t="s">
         <v>167</v>
       </c>
@@ -6568,7 +6513,7 @@
       </c>
       <c r="K76" s="45"/>
     </row>
-    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6603,7 +6548,7 @@
       </c>
       <c r="K77" s="45"/>
     </row>
-    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6638,7 +6583,7 @@
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6673,7 +6618,7 @@
       </c>
       <c r="K79" s="45"/>
     </row>
-    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6708,7 +6653,7 @@
       </c>
       <c r="K80" s="45"/>
     </row>
-    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6743,7 +6688,7 @@
       </c>
       <c r="K81" s="45"/>
     </row>
-    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6778,7 +6723,7 @@
       </c>
       <c r="K82" s="45"/>
     </row>
-    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="18" t="s">
         <v>182</v>
       </c>
@@ -6813,7 +6758,7 @@
       </c>
       <c r="K83" s="45"/>
     </row>
-    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6848,7 +6793,7 @@
       </c>
       <c r="K84" s="45"/>
     </row>
-    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6883,7 +6828,7 @@
       </c>
       <c r="K85" s="45"/>
     </row>
-    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6918,7 +6863,7 @@
       </c>
       <c r="K86" s="45"/>
     </row>
-    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6953,7 +6898,7 @@
       </c>
       <c r="K87" s="45"/>
     </row>
-    <row r="88" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="18" t="s">
         <v>194</v>
       </c>
@@ -6988,7 +6933,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7023,7 +6968,7 @@
       </c>
       <c r="K89" s="46"/>
     </row>
-    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7058,7 +7003,7 @@
       </c>
       <c r="K90" s="46"/>
     </row>
-    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="18" t="s">
         <v>200</v>
       </c>
@@ -7093,7 +7038,7 @@
       </c>
       <c r="K91" s="46"/>
     </row>
-    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7128,7 +7073,7 @@
       </c>
       <c r="K92" s="46"/>
     </row>
-    <row r="93" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="18" t="s">
         <v>204</v>
       </c>
@@ -7163,7 +7108,7 @@
       </c>
       <c r="K93" s="46"/>
     </row>
-    <row r="94" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7198,7 +7143,7 @@
       </c>
       <c r="K94" s="46"/>
     </row>
-    <row r="95" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7233,7 +7178,7 @@
       </c>
       <c r="K95" s="46"/>
     </row>
-    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
         <v>75</v>
@@ -7262,7 +7207,7 @@
       </c>
       <c r="K96" s="46"/>
     </row>
-    <row r="97" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
         <v>76</v>
@@ -7291,7 +7236,7 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
         <v>77</v>
@@ -7320,7 +7265,7 @@
       </c>
       <c r="K98" s="46"/>
     </row>
-    <row r="99" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
         <v>78</v>
@@ -7349,7 +7294,7 @@
       </c>
       <c r="K99" s="46"/>
     </row>
-    <row r="100" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
         <v>79</v>
@@ -7380,7 +7325,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="101" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
         <v>80</v>
@@ -7409,7 +7354,7 @@
       </c>
       <c r="K101" s="47"/>
     </row>
-    <row r="102" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
         <v>81</v>
@@ -7438,7 +7383,7 @@
       </c>
       <c r="K102" s="47"/>
     </row>
-    <row r="103" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
         <v>82</v>
@@ -7467,7 +7412,7 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
         <v>83</v>
@@ -7496,7 +7441,7 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="3:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="3:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
         <v>84</v>
@@ -7525,7 +7470,7 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
         <v>85</v>
@@ -7554,7 +7499,7 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
         <v>86</v>
@@ -7583,7 +7528,7 @@
       </c>
       <c r="K107" s="47"/>
     </row>
-    <row r="108" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
         <v>87</v>
@@ -7612,7 +7557,7 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
         <v>88</v>
@@ -7641,7 +7586,7 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
         <v>89</v>
@@ -7670,7 +7615,7 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
         <v>90</v>
@@ -7699,7 +7644,7 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
         <v>91</v>
@@ -7728,7 +7673,7 @@
       </c>
       <c r="K112" s="47"/>
     </row>
-    <row r="113" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
         <v>92</v>
@@ -7757,7 +7702,7 @@
       </c>
       <c r="K113" s="47"/>
     </row>
-    <row r="114" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
         <v>93</v>
@@ -7786,7 +7731,7 @@
       </c>
       <c r="K114" s="47"/>
     </row>
-    <row r="115" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
         <v>94</v>
@@ -7815,7 +7760,7 @@
       </c>
       <c r="K115" s="47"/>
     </row>
-    <row r="116" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
         <v>95</v>
@@ -7844,7 +7789,7 @@
       </c>
       <c r="K116" s="47"/>
     </row>
-    <row r="117" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
         <v>96</v>
@@ -7873,7 +7818,7 @@
       </c>
       <c r="K117" s="47"/>
     </row>
-    <row r="118" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
         <v>97</v>
@@ -7902,7 +7847,7 @@
       </c>
       <c r="K118" s="47"/>
     </row>
-    <row r="119" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
         <v>98</v>
@@ -7931,7 +7876,7 @@
       </c>
       <c r="K119" s="47"/>
     </row>
-    <row r="120" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
         <v>99</v>
@@ -7960,7 +7905,7 @@
       </c>
       <c r="K120" s="47"/>
     </row>
-    <row r="121" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
         <v>100</v>
@@ -7988,7 +7933,7 @@
       </c>
       <c r="K121" s="47"/>
     </row>
-    <row r="122" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
         <v>101</v>
@@ -8016,7 +7961,7 @@
       </c>
       <c r="K122" s="47"/>
     </row>
-    <row r="123" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
         <v>102</v>
@@ -8044,7 +7989,7 @@
       </c>
       <c r="K123" s="47"/>
     </row>
-    <row r="124" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
         <v>103</v>
@@ -8072,7 +8017,7 @@
       </c>
       <c r="K124" s="47"/>
     </row>
-    <row r="125" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
         <v>104</v>
@@ -8100,7 +8045,7 @@
       </c>
       <c r="K125" s="47"/>
     </row>
-    <row r="126" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
         <v>105</v>
@@ -8128,7 +8073,7 @@
       </c>
       <c r="K126" s="47"/>
     </row>
-    <row r="127" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
         <v>106</v>
@@ -8156,7 +8101,7 @@
       </c>
       <c r="K127" s="47"/>
     </row>
-    <row r="128" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
         <v>107</v>
@@ -8184,7 +8129,7 @@
       </c>
       <c r="K128" s="47"/>
     </row>
-    <row r="129" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
         <v>108</v>
@@ -8212,7 +8157,7 @@
       </c>
       <c r="K129" s="47"/>
     </row>
-    <row r="130" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
         <v>109</v>
@@ -8240,7 +8185,7 @@
       </c>
       <c r="K130" s="47"/>
     </row>
-    <row r="131" spans="3:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="3:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
         <v>110</v>
@@ -8268,7 +8213,7 @@
       </c>
       <c r="K131" s="47"/>
     </row>
-    <row r="132" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
         <v>111</v>
@@ -8296,7 +8241,7 @@
       </c>
       <c r="K132" s="47"/>
     </row>
-    <row r="133" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
         <v>112</v>
@@ -8324,7 +8269,7 @@
       </c>
       <c r="K133" s="47"/>
     </row>
-    <row r="134" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
         <v>113</v>
@@ -8354,7 +8299,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
         <v>114</v>
@@ -8382,7 +8327,7 @@
       </c>
       <c r="K135" s="46"/>
     </row>
-    <row r="136" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
         <v>115</v>
@@ -8410,7 +8355,7 @@
       </c>
       <c r="K136" s="46"/>
     </row>
-    <row r="137" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
         <v>116</v>
@@ -8438,7 +8383,7 @@
       </c>
       <c r="K137" s="46"/>
     </row>
-    <row r="138" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
         <v>117</v>
@@ -8466,7 +8411,7 @@
       </c>
       <c r="K138" s="46"/>
     </row>
-    <row r="139" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
         <v>118</v>
@@ -8494,7 +8439,7 @@
       </c>
       <c r="K139" s="46"/>
     </row>
-    <row r="140" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
         <v>119</v>
@@ -8525,7 +8470,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="141" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
         <v>120</v>
@@ -8556,7 +8501,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="142" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
         <v>121</v>

</xml_diff>

<commit_message>
Fix thickness reference: Bun thickness and Min Sheet thickness
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90AA8A06-8E0F-4484-B908-271C8F7F655C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -4309,7 +4309,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:K142"/>
@@ -4625,41 +4625,40 @@
       <c r="K22" s="44"/>
     </row>
     <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="18" t="e">
+      <c r="A23" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B23" s="18" t="s">
-        <v>48</v>
-      </c>
       <c r="C23" s="29">
-        <f>IF(E23&lt;&gt;"",SUBTOTAL(103,E$22:E23),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="E23" s="37" t="s">
-        <v>49</v>
+        <v>60</v>
+      </c>
+      <c r="E23" s="31" t="s">
+        <v>61</v>
       </c>
       <c r="F23" s="32" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="G23" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J23" s="35">
         <f>+IFERROR(VLOOKUP(E23,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43040</v>
-      </c>
-      <c r="K23" s="44"/>
-    </row>
-    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>43720</v>
+      </c>
+      <c r="K23" s="45"/>
+    </row>
+    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4668,7 +4667,7 @@
       </c>
       <c r="C24" s="29">
         <f>IF(E24&lt;&gt;"",SUBTOTAL(103,E$22:E24),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>44</v>
@@ -4694,7 +4693,7 @@
       </c>
       <c r="K24" s="44"/>
     </row>
-    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4703,7 +4702,7 @@
       </c>
       <c r="C25" s="29">
         <f>IF(E25&lt;&gt;"",SUBTOTAL(103,E$22:E25),"")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>44</v>
@@ -4730,24 +4729,24 @@
       <c r="K25" s="44"/>
     </row>
     <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B26" s="18" t="e">
+      <c r="A26" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>76</v>
       </c>
       <c r="C26" s="29">
         <f>IF(E26&lt;&gt;"",SUBTOTAL(103,E$22:E26),"")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D26" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E26" s="37" t="s">
-        <v>57</v>
+      <c r="E26" s="31" t="s">
+        <v>77</v>
       </c>
       <c r="F26" s="32" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G26" s="33" t="s">
         <v>46</v>
@@ -4756,67 +4755,68 @@
         <v>47</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J26" s="35">
         <f>+IFERROR(VLOOKUP(E26,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43356</v>
+        <v>43867</v>
       </c>
       <c r="K26" s="45"/>
     </row>
     <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B27" s="18" t="e">
+      <c r="A27" s="18" t="e">
         <v>#N/A</v>
       </c>
+      <c r="B27" s="18" t="s">
+        <v>78</v>
+      </c>
       <c r="C27" s="29">
-        <v>1</v>
+        <f>IF(E27&lt;&gt;"",SUBTOTAL(103,E$22:E27),"")</f>
+        <v>4</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="F27" s="32" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="G27" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I27" s="34" t="s">
         <v>50</v>
       </c>
       <c r="J27" s="35">
         <f>+IFERROR(VLOOKUP(E27,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43720</v>
+        <v>43871</v>
       </c>
       <c r="K27" s="45"/>
     </row>
     <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" s="18" t="e">
+      <c r="A28" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>84</v>
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="F28" s="32" t="s">
-        <v>63</v>
+      <c r="E28" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="F28" s="39" t="s">
+        <v>84</v>
       </c>
       <c r="G28" s="33" t="s">
         <v>46</v>
@@ -4825,68 +4825,68 @@
         <v>47</v>
       </c>
       <c r="I28" s="34" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J28" s="35">
         <f>+IFERROR(VLOOKUP(E28,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43808</v>
+        <v>43875</v>
       </c>
       <c r="K28" s="45"/>
     </row>
     <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="18" t="s">
-        <v>65</v>
+      <c r="A29" s="18" t="e">
+        <v>#N/A</v>
       </c>
       <c r="B29" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="F29" s="32" t="s">
-        <v>65</v>
+        <v>104</v>
       </c>
       <c r="G29" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H29" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I29" s="34" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J29" s="35">
         <f>+IFERROR(VLOOKUP(E29,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43803</v>
+        <v>43875</v>
       </c>
       <c r="K29" s="45"/>
     </row>
     <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B30" s="18" t="e">
+      <c r="A30" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>134</v>
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E30" s="31" t="s">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="F30" s="32" t="s">
-        <v>67</v>
+        <v>134</v>
       </c>
       <c r="G30" s="33" t="s">
         <v>46</v>
@@ -4895,15 +4895,15 @@
         <v>62</v>
       </c>
       <c r="I30" s="34" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J30" s="35">
         <f>+IFERROR(VLOOKUP(E30,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43867</v>
+        <v>44256</v>
       </c>
       <c r="K30" s="45"/>
     </row>
-    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="K31" s="45"/>
     </row>
-    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -4974,37 +4974,37 @@
       <c r="K32" s="45"/>
     </row>
     <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="18" t="e">
+      <c r="A33" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="B33" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>76</v>
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D33" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="F33" s="32" t="s">
-        <v>76</v>
+        <v>183</v>
+      </c>
+      <c r="F33" s="34" t="s">
+        <v>182</v>
       </c>
       <c r="G33" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I33" s="34" t="s">
         <v>50</v>
       </c>
       <c r="J33" s="35">
         <f>+IFERROR(VLOOKUP(E33,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43867</v>
+        <v>44993</v>
       </c>
       <c r="K33" s="45"/>
     </row>
@@ -5013,37 +5013,37 @@
         <v>#N/A</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="F34" s="32" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="G34" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H34" s="33" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="I34" s="34" t="s">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="J34" s="35">
         <f>+IFERROR(VLOOKUP(E34,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43871</v>
+        <v>43672</v>
       </c>
       <c r="K34" s="45"/>
     </row>
-    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5079,24 +5079,20 @@
       <c r="K35" s="45"/>
     </row>
     <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="18" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="B36" s="18" t="s">
-        <v>82</v>
-      </c>
+      <c r="A36"/>
+      <c r="B36"/>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E36" s="38" t="s">
-        <v>83</v>
-      </c>
-      <c r="F36" s="39" t="s">
-        <v>82</v>
+      <c r="E36" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="F36" s="32" t="s">
+        <v>260</v>
       </c>
       <c r="G36" s="33" t="s">
         <v>46</v>
@@ -5105,46 +5101,46 @@
         <v>47</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="J36" s="35">
+        <v>94</v>
+      </c>
+      <c r="J36" s="35" t="str">
         <f>+IFERROR(VLOOKUP(E36,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
-      </c>
-      <c r="K36" s="45"/>
+        <v>29/09/2025</v>
+      </c>
+      <c r="K36" s="47"/>
     </row>
     <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="18" t="e">
+      <c r="A37" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B37" s="18" t="s">
-        <v>84</v>
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="E37" s="38" t="s">
-        <v>85</v>
-      </c>
-      <c r="F37" s="39" t="s">
-        <v>84</v>
+        <v>60</v>
+      </c>
+      <c r="E37" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="F37" s="32" t="s">
+        <v>119</v>
       </c>
       <c r="G37" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>50</v>
+        <v>121</v>
       </c>
       <c r="J37" s="35">
         <f>+IFERROR(VLOOKUP(E37,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
+        <v>44043</v>
       </c>
       <c r="K37" s="45"/>
     </row>
@@ -5152,38 +5148,38 @@
       <c r="A38" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B38" s="18" t="s">
-        <v>86</v>
+      <c r="B38" s="18" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D38" s="30" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E38" s="31" t="s">
-        <v>87</v>
+        <v>136</v>
       </c>
       <c r="F38" s="32" t="s">
-        <v>86</v>
+        <v>137</v>
       </c>
       <c r="G38" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H38" s="33" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="I38" s="34" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="J38" s="35">
         <f>+IFERROR(VLOOKUP(E38,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43903</v>
+        <v>44312</v>
       </c>
       <c r="K38" s="45"/>
     </row>
-    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5192,7 +5188,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5223,33 +5219,33 @@
         <v>#N/A</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E40" s="31" t="s">
-        <v>93</v>
+        <v>162</v>
       </c>
       <c r="F40" s="32" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="G40" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H40" s="33" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="I40" s="34" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="J40" s="35">
         <f>+IFERROR(VLOOKUP(E40,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43672</v>
+        <v>44630</v>
       </c>
       <c r="K40" s="45"/>
     </row>
@@ -5258,37 +5254,37 @@
         <v>#N/A</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D41" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>96</v>
+        <v>166</v>
       </c>
       <c r="F41" s="32" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="G41" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H41" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I41" s="34" t="s">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="J41" s="35">
         <f>+IFERROR(VLOOKUP(E41,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43846</v>
+        <v>44634</v>
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5297,7 +5293,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5323,7 +5319,7 @@
       </c>
       <c r="K42" s="45"/>
     </row>
-    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5332,7 +5328,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5363,33 +5359,33 @@
         <v>#N/A</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>101</v>
+        <v>171</v>
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D44" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E44" s="31" t="s">
-        <v>102</v>
-      </c>
-      <c r="F44" s="32" t="s">
-        <v>101</v>
+        <v>172</v>
+      </c>
+      <c r="F44" s="34" t="s">
+        <v>171</v>
       </c>
       <c r="G44" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H44" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I44" s="34" t="s">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="J44" s="35">
         <f>+IFERROR(VLOOKUP(E44,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43867</v>
+        <v>44707</v>
       </c>
       <c r="K44" s="45"/>
     </row>
@@ -5397,56 +5393,56 @@
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B45" s="18" t="e">
-        <v>#N/A</v>
+      <c r="B45" s="18" t="s">
+        <v>48</v>
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D45" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E45" s="31" t="s">
-        <v>103</v>
+        <v>44</v>
+      </c>
+      <c r="E45" s="37" t="s">
+        <v>49</v>
       </c>
       <c r="F45" s="32" t="s">
-        <v>104</v>
+        <v>48</v>
       </c>
       <c r="G45" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H45" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I45" s="34" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="J45" s="35">
         <f>+IFERROR(VLOOKUP(E45,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
-      </c>
-      <c r="K45" s="45"/>
+        <v>43040</v>
+      </c>
+      <c r="K45" s="44"/>
     </row>
     <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="B46" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E46" s="38" t="s">
-        <v>106</v>
-      </c>
-      <c r="F46" s="39" t="s">
-        <v>105</v>
+      <c r="E46" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="F46" s="32" t="s">
+        <v>56</v>
       </c>
       <c r="G46" s="33" t="s">
         <v>46</v>
@@ -5459,11 +5455,11 @@
       </c>
       <c r="J46" s="35">
         <f>+IFERROR(VLOOKUP(E46,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
+        <v>43356</v>
       </c>
       <c r="K46" s="45"/>
     </row>
-    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5472,7 +5468,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5499,24 +5495,24 @@
       <c r="K47" s="45"/>
     </row>
     <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="18" t="e">
+      <c r="A48" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B48" s="18" t="s">
-        <v>109</v>
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E48" s="37" t="s">
-        <v>110</v>
+      <c r="E48" s="31" t="s">
+        <v>64</v>
       </c>
       <c r="F48" s="32" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="G48" s="33" t="s">
         <v>46</v>
@@ -5529,11 +5525,11 @@
       </c>
       <c r="J48" s="35">
         <f>+IFERROR(VLOOKUP(E48,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43844</v>
+        <v>43808</v>
       </c>
       <c r="K48" s="45"/>
     </row>
-    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="18" t="s">
         <v>111</v>
       </c>
@@ -5542,7 +5538,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5568,7 +5564,7 @@
       </c>
       <c r="K49" s="45"/>
     </row>
-    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5577,7 +5573,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5604,41 +5600,41 @@
       <c r="K50" s="45"/>
     </row>
     <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="18" t="e">
+      <c r="A51" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B51" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B51" s="18" t="s">
-        <v>115</v>
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="D51" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="F51" s="32" t="s">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="G51" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H51" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I51" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J51" s="35">
         <f>+IFERROR(VLOOKUP(E51,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44029</v>
+        <v>43803</v>
       </c>
       <c r="K51" s="45"/>
     </row>
-    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5647,7 +5643,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5675,23 +5671,23 @@
     </row>
     <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
       <c r="B53" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E53" s="31" t="s">
-        <v>120</v>
+        <v>68</v>
       </c>
       <c r="F53" s="32" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
       <c r="G53" s="33" t="s">
         <v>46</v>
@@ -5700,15 +5696,15 @@
         <v>62</v>
       </c>
       <c r="I53" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J53" s="35">
         <f>+IFERROR(VLOOKUP(E53,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44043</v>
+        <v>43867</v>
       </c>
       <c r="K53" s="45"/>
     </row>
-    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5717,7 +5713,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5747,38 +5743,38 @@
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B55" s="18" t="e">
-        <v>#N/A</v>
+      <c r="B55" s="18" t="s">
+        <v>82</v>
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E55" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="F55" s="32" t="s">
-        <v>125</v>
+        <v>44</v>
+      </c>
+      <c r="E55" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="F55" s="39" t="s">
+        <v>82</v>
       </c>
       <c r="G55" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H55" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I55" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J55" s="35">
         <f>+IFERROR(VLOOKUP(E55,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44077</v>
+        <v>43875</v>
       </c>
       <c r="K55" s="45"/>
     </row>
-    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5787,7 +5783,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5818,20 +5814,20 @@
         <v>#N/A</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>128</v>
+        <v>95</v>
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>44</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="F57" s="32" t="s">
-        <v>128</v>
+        <v>95</v>
       </c>
       <c r="G57" s="33" t="s">
         <v>46</v>
@@ -5844,11 +5840,11 @@
       </c>
       <c r="J57" s="35">
         <f>+IFERROR(VLOOKUP(E57,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44118</v>
+        <v>43846</v>
       </c>
       <c r="K57" s="45"/>
     </row>
-    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5857,7 +5853,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5883,7 +5879,7 @@
       </c>
       <c r="K58" s="45"/>
     </row>
-    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5892,7 +5888,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5923,72 +5919,72 @@
         <v>#N/A</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D60" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E60" s="31" t="s">
-        <v>135</v>
+        <v>102</v>
       </c>
       <c r="F60" s="32" t="s">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="G60" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H60" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I60" s="34" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="J60" s="35">
         <f>+IFERROR(VLOOKUP(E60,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44256</v>
+        <v>43867</v>
       </c>
       <c r="K60" s="45"/>
     </row>
     <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="18" t="e">
-        <v>#N/A</v>
+      <c r="A61" s="18" t="s">
+        <v>105</v>
       </c>
       <c r="B61" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="D61" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E61" s="31" t="s">
-        <v>136</v>
-      </c>
-      <c r="F61" s="32" t="s">
-        <v>137</v>
+        <v>44</v>
+      </c>
+      <c r="E61" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="F61" s="39" t="s">
+        <v>105</v>
       </c>
       <c r="G61" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H61" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I61" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J61" s="35">
         <f>+IFERROR(VLOOKUP(E61,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44312</v>
+        <v>43875</v>
       </c>
       <c r="K61" s="45"/>
     </row>
-    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="18" t="s">
         <v>138</v>
       </c>
@@ -5997,7 +5993,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6023,7 +6019,7 @@
       </c>
       <c r="K62" s="45"/>
     </row>
-    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6032,7 +6028,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6058,7 +6054,7 @@
       </c>
       <c r="K63" s="45"/>
     </row>
-    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6067,7 +6063,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6093,7 +6089,7 @@
       </c>
       <c r="K64" s="45"/>
     </row>
-    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="18" t="s">
         <v>145</v>
       </c>
@@ -6102,7 +6098,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6133,37 +6129,37 @@
         <v>#N/A</v>
       </c>
       <c r="B66" s="18" t="s">
-        <v>147</v>
+        <v>109</v>
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="D66" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E66" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="F66" s="39" t="s">
-        <v>147</v>
+        <v>44</v>
+      </c>
+      <c r="E66" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F66" s="32" t="s">
+        <v>109</v>
       </c>
       <c r="G66" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H66" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I66" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J66" s="35">
         <f>+IFERROR(VLOOKUP(E66,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44516</v>
+        <v>43844</v>
       </c>
       <c r="K66" s="45"/>
     </row>
-    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6172,7 +6168,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6198,7 +6194,7 @@
       </c>
       <c r="K67" s="45"/>
     </row>
-    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="18" t="s">
         <v>151</v>
       </c>
@@ -6207,7 +6203,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6233,7 +6229,7 @@
       </c>
       <c r="K68" s="45"/>
     </row>
-    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6242,7 +6238,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6273,20 +6269,20 @@
         <v>#N/A</v>
       </c>
       <c r="B70" s="18" t="s">
-        <v>155</v>
+        <v>115</v>
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E70" s="31" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="F70" s="32" t="s">
-        <v>155</v>
+        <v>115</v>
       </c>
       <c r="G70" s="33" t="s">
         <v>46</v>
@@ -6299,29 +6295,29 @@
       </c>
       <c r="J70" s="35">
         <f>+IFERROR(VLOOKUP(E70,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44603</v>
+        <v>44029</v>
       </c>
       <c r="K70" s="45"/>
     </row>
     <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="18" t="s">
-        <v>157</v>
+      <c r="A71" s="18" t="e">
+        <v>#N/A</v>
       </c>
       <c r="B71" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E71" s="31" t="s">
-        <v>158</v>
+        <v>124</v>
       </c>
       <c r="F71" s="32" t="s">
-        <v>157</v>
+        <v>125</v>
       </c>
       <c r="G71" s="33" t="s">
         <v>46</v>
@@ -6334,7 +6330,7 @@
       </c>
       <c r="J71" s="35">
         <f>+IFERROR(VLOOKUP(E71,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44610</v>
+        <v>44077</v>
       </c>
       <c r="K71" s="45"/>
     </row>
@@ -6343,20 +6339,20 @@
         <v>#N/A</v>
       </c>
       <c r="B72" s="18" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
       </c>
       <c r="E72" s="31" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="F72" s="32" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="G72" s="33" t="s">
         <v>46</v>
@@ -6369,7 +6365,7 @@
       </c>
       <c r="J72" s="35">
         <f>+IFERROR(VLOOKUP(E72,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44630</v>
+        <v>44118</v>
       </c>
       <c r="K72" s="45"/>
     </row>
@@ -6378,20 +6374,20 @@
         <v>#N/A</v>
       </c>
       <c r="B73" s="18" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E73" s="31" t="s">
-        <v>162</v>
-      </c>
-      <c r="F73" s="32" t="s">
-        <v>161</v>
+        <v>148</v>
+      </c>
+      <c r="F73" s="39" t="s">
+        <v>147</v>
       </c>
       <c r="G73" s="33" t="s">
         <v>46</v>
@@ -6400,68 +6396,68 @@
         <v>62</v>
       </c>
       <c r="I73" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J73" s="35">
         <f>+IFERROR(VLOOKUP(E73,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44630</v>
+        <v>44516</v>
       </c>
       <c r="K73" s="45"/>
     </row>
     <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="B74" s="18" t="e">
+      <c r="A74" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>155</v>
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="D74" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E74" s="31" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="F74" s="32" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="G74" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H74" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I74" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J74" s="35">
         <f>+IFERROR(VLOOKUP(E74,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44634</v>
+        <v>44603</v>
       </c>
       <c r="K74" s="45"/>
     </row>
     <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="18" t="e">
+      <c r="A75" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B75" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B75" s="18" t="s">
-        <v>165</v>
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E75" s="31" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="F75" s="32" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="G75" s="33" t="s">
         <v>46</v>
@@ -6470,15 +6466,15 @@
         <v>62</v>
       </c>
       <c r="I75" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J75" s="35">
         <f>+IFERROR(VLOOKUP(E75,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44634</v>
+        <v>44610</v>
       </c>
       <c r="K75" s="45"/>
     </row>
-    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="18" t="s">
         <v>167</v>
       </c>
@@ -6487,7 +6483,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6513,7 +6509,7 @@
       </c>
       <c r="K76" s="45"/>
     </row>
-    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6522,7 +6518,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6553,37 +6549,37 @@
         <v>#N/A</v>
       </c>
       <c r="B78" s="18" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="D78" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E78" s="31" t="s">
-        <v>172</v>
-      </c>
-      <c r="F78" s="34" t="s">
-        <v>171</v>
+        <v>160</v>
+      </c>
+      <c r="F78" s="32" t="s">
+        <v>159</v>
       </c>
       <c r="G78" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H78" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I78" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J78" s="35">
         <f>+IFERROR(VLOOKUP(E78,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44707</v>
+        <v>44630</v>
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6592,7 +6588,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6618,7 +6614,7 @@
       </c>
       <c r="K79" s="45"/>
     </row>
-    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6627,7 +6623,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6653,7 +6649,7 @@
       </c>
       <c r="K80" s="45"/>
     </row>
-    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6662,7 +6658,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6688,7 +6684,7 @@
       </c>
       <c r="K81" s="45"/>
     </row>
-    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6697,7 +6693,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6725,40 +6721,40 @@
     </row>
     <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="18" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
       <c r="B83" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="D83" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E83" s="31" t="s">
-        <v>183</v>
-      </c>
-      <c r="F83" s="34" t="s">
-        <v>182</v>
+        <v>164</v>
+      </c>
+      <c r="F83" s="32" t="s">
+        <v>163</v>
       </c>
       <c r="G83" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H83" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I83" s="34" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="J83" s="35">
         <f>+IFERROR(VLOOKUP(E83,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44993</v>
+        <v>44634</v>
       </c>
       <c r="K83" s="45"/>
     </row>
-    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6767,7 +6763,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6793,7 +6789,7 @@
       </c>
       <c r="K84" s="45"/>
     </row>
-    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6802,7 +6798,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6828,7 +6824,7 @@
       </c>
       <c r="K85" s="45"/>
     </row>
-    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6837,7 +6833,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6863,7 +6859,7 @@
       </c>
       <c r="K86" s="45"/>
     </row>
-    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6872,7 +6868,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6898,7 +6894,7 @@
       </c>
       <c r="K87" s="45"/>
     </row>
-    <row r="88" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="18" t="s">
         <v>194</v>
       </c>
@@ -6907,7 +6903,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6933,7 +6929,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6942,7 +6938,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -6968,7 +6964,7 @@
       </c>
       <c r="K89" s="46"/>
     </row>
-    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6977,7 +6973,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7012,7 +7008,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>60</v>
@@ -7038,7 +7034,7 @@
       </c>
       <c r="K91" s="46"/>
     </row>
-    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7047,7 +7043,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7073,7 +7069,7 @@
       </c>
       <c r="K92" s="46"/>
     </row>
-    <row r="93" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="18" t="s">
         <v>204</v>
       </c>
@@ -7082,7 +7078,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7108,7 +7104,7 @@
       </c>
       <c r="K93" s="46"/>
     </row>
-    <row r="94" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7117,7 +7113,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7143,7 +7139,7 @@
       </c>
       <c r="K94" s="46"/>
     </row>
-    <row r="95" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7152,7 +7148,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7178,10 +7174,10 @@
       </c>
       <c r="K95" s="46"/>
     </row>
-    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7207,10 +7203,10 @@
       </c>
       <c r="K96" s="46"/>
     </row>
-    <row r="97" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7236,10 +7232,10 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7265,10 +7261,10 @@
       </c>
       <c r="K98" s="46"/>
     </row>
-    <row r="99" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7294,10 +7290,10 @@
       </c>
       <c r="K99" s="46"/>
     </row>
-    <row r="100" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7325,10 +7321,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="101" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7357,7 +7353,7 @@
     <row r="102" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>72</v>
@@ -7383,10 +7379,10 @@
       </c>
       <c r="K102" s="47"/>
     </row>
-    <row r="103" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7412,10 +7408,10 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7441,10 +7437,10 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="3:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="3:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7470,10 +7466,10 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7499,10 +7495,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7528,10 +7524,10 @@
       </c>
       <c r="K107" s="47"/>
     </row>
-    <row r="108" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7557,10 +7553,10 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7586,10 +7582,10 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7615,10 +7611,10 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7644,10 +7640,10 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7673,10 +7669,10 @@
       </c>
       <c r="K112" s="47"/>
     </row>
-    <row r="113" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>92</v>
+        <v>35</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7702,10 +7698,10 @@
       </c>
       <c r="K113" s="47"/>
     </row>
-    <row r="114" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7731,10 +7727,10 @@
       </c>
       <c r="K114" s="47"/>
     </row>
-    <row r="115" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7760,10 +7756,10 @@
       </c>
       <c r="K115" s="47"/>
     </row>
-    <row r="116" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7789,10 +7785,10 @@
       </c>
       <c r="K116" s="47"/>
     </row>
-    <row r="117" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>96</v>
+        <v>35</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7818,10 +7814,10 @@
       </c>
       <c r="K117" s="47"/>
     </row>
-    <row r="118" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>97</v>
+        <v>35</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7847,39 +7843,45 @@
       </c>
       <c r="K118" s="47"/>
     </row>
-    <row r="119" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="B119" s="18" t="s">
+        <v>86</v>
+      </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>98</v>
+        <v>36</v>
       </c>
       <c r="D119" s="30" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="E119" s="31" t="s">
-        <v>259</v>
+        <v>87</v>
       </c>
       <c r="F119" s="32" t="s">
-        <v>260</v>
+        <v>86</v>
       </c>
       <c r="G119" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H119" s="33" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="I119" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="J119" s="35" t="str">
+        <v>88</v>
+      </c>
+      <c r="J119" s="35">
         <f>+IFERROR(VLOOKUP(E119,[1]Sheet1!C:H,6,0),"")</f>
-        <v>29/09/2025</v>
-      </c>
-      <c r="K119" s="47"/>
-    </row>
-    <row r="120" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>43903</v>
+      </c>
+      <c r="K119" s="45"/>
+    </row>
+    <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>99</v>
+        <v>36</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7905,10 +7907,10 @@
       </c>
       <c r="K120" s="47"/>
     </row>
-    <row r="121" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7933,10 +7935,10 @@
       </c>
       <c r="K121" s="47"/>
     </row>
-    <row r="122" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -7961,10 +7963,10 @@
       </c>
       <c r="K122" s="47"/>
     </row>
-    <row r="123" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -7989,10 +7991,10 @@
       </c>
       <c r="K123" s="47"/>
     </row>
-    <row r="124" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>103</v>
+        <v>36</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8017,10 +8019,10 @@
       </c>
       <c r="K124" s="47"/>
     </row>
-    <row r="125" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>104</v>
+        <v>36</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8045,10 +8047,10 @@
       </c>
       <c r="K125" s="47"/>
     </row>
-    <row r="126" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8073,10 +8075,10 @@
       </c>
       <c r="K126" s="47"/>
     </row>
-    <row r="127" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>106</v>
+        <v>36</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8101,10 +8103,10 @@
       </c>
       <c r="K127" s="47"/>
     </row>
-    <row r="128" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>107</v>
+        <v>36</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8129,10 +8131,10 @@
       </c>
       <c r="K128" s="47"/>
     </row>
-    <row r="129" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8157,10 +8159,10 @@
       </c>
       <c r="K129" s="47"/>
     </row>
-    <row r="130" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>109</v>
+        <v>36</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8185,10 +8187,10 @@
       </c>
       <c r="K130" s="47"/>
     </row>
-    <row r="131" spans="3:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8213,10 +8215,10 @@
       </c>
       <c r="K131" s="47"/>
     </row>
-    <row r="132" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>111</v>
+        <v>36</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8241,10 +8243,10 @@
       </c>
       <c r="K132" s="47"/>
     </row>
-    <row r="133" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>112</v>
+        <v>36</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8269,10 +8271,10 @@
       </c>
       <c r="K133" s="47"/>
     </row>
-    <row r="134" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>113</v>
+        <v>36</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8299,10 +8301,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8327,10 +8329,10 @@
       </c>
       <c r="K135" s="46"/>
     </row>
-    <row r="136" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>115</v>
+        <v>36</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8355,10 +8357,10 @@
       </c>
       <c r="K136" s="46"/>
     </row>
-    <row r="137" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>116</v>
+        <v>36</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8383,10 +8385,10 @@
       </c>
       <c r="K137" s="46"/>
     </row>
-    <row r="138" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>117</v>
+        <v>36</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8411,10 +8413,10 @@
       </c>
       <c r="K138" s="46"/>
     </row>
-    <row r="139" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>118</v>
+        <v>36</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8439,10 +8441,10 @@
       </c>
       <c r="K139" s="46"/>
     </row>
-    <row r="140" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>119</v>
+        <v>36</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8470,10 +8472,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="141" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>120</v>
+        <v>36</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8501,10 +8503,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="142" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>121</v>
+        <v>36</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8533,7 +8535,21 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A21:FL142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}"/>
+  <autoFilter ref="A21:FL142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Group Leader"/>
+        <filter val="Junior Technician"/>
+        <filter val="Operator"/>
+        <filter val="Skilled worker"/>
+        <filter val="Supervisor"/>
+        <filter val="Team Leader"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A22:K119">
+      <sortCondition descending="1" ref="I21:I142"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>

<commit_message>
Enhance NG recording: support multiple errors and dropdown selection
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90AA8A06-8E0F-4484-B908-271C8F7F655C}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFCFBBC9-FCD5-4844-B74F-B34C4805BF99}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -1482,7 +1482,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1504,6 +1504,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1565,7 +1571,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1699,6 +1705,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -4589,74 +4604,71 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="C22" s="29">
         <f>IF(E22&lt;&gt;"",SUBTOTAL(103,E$22:E22),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="F22" s="32" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="G22" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H22" s="33" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="I22" s="34" t="s">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="J22" s="35">
         <f>+IFERROR(VLOOKUP(E22,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44118</v>
-      </c>
-      <c r="K22" s="44"/>
-    </row>
-    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B23" s="18" t="e">
-        <v>#N/A</v>
-      </c>
+        <v>43672</v>
+      </c>
+      <c r="K22" s="45"/>
+    </row>
+    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23"/>
+      <c r="B23"/>
       <c r="C23" s="29">
-        <v>1</v>
+        <f>IF(E23&lt;&gt;"",SUBTOTAL(103,E$22:E23),"")</f>
+        <v>0</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="E23" s="31" t="s">
-        <v>61</v>
+        <v>222</v>
       </c>
       <c r="F23" s="32" t="s">
-        <v>59</v>
+        <v>223</v>
       </c>
       <c r="G23" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="J23" s="35">
+        <v>224</v>
+      </c>
+      <c r="J23" s="35" t="str">
         <f>+IFERROR(VLOOKUP(E23,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43720</v>
-      </c>
-      <c r="K23" s="45"/>
+        <v>30/09/2024</v>
+      </c>
+      <c r="K23" s="47"/>
     </row>
     <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="e">
@@ -4667,7 +4679,7 @@
       </c>
       <c r="C24" s="29">
         <f>IF(E24&lt;&gt;"",SUBTOTAL(103,E$22:E24),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>44</v>
@@ -4702,7 +4714,7 @@
       </c>
       <c r="C25" s="29">
         <f>IF(E25&lt;&gt;"",SUBTOTAL(103,E$22:E25),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>44</v>
@@ -4728,73 +4740,72 @@
       </c>
       <c r="K25" s="44"/>
     </row>
-    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="C26" s="29">
         <f>IF(E26&lt;&gt;"",SUBTOTAL(103,E$22:E26),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F26" s="32" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G26" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H26" s="33" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="J26" s="35">
         <f>+IFERROR(VLOOKUP(E26,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43867</v>
+        <v>43903</v>
       </c>
       <c r="K26" s="45"/>
     </row>
     <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="18" t="e">
+      <c r="A27" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B27" s="18" t="s">
-        <v>78</v>
-      </c>
       <c r="C27" s="29">
-        <f>IF(E27&lt;&gt;"",SUBTOTAL(103,E$22:E27),"")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="F27" s="32" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="G27" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I27" s="34" t="s">
         <v>50</v>
       </c>
       <c r="J27" s="35">
         <f>+IFERROR(VLOOKUP(E27,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43871</v>
+        <v>43720</v>
       </c>
       <c r="K27" s="45"/>
     </row>
@@ -4802,27 +4813,27 @@
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>84</v>
+      <c r="B28" s="18" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="E28" s="38" t="s">
-        <v>85</v>
-      </c>
-      <c r="F28" s="39" t="s">
-        <v>84</v>
+        <v>60</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="F28" s="32" t="s">
+        <v>104</v>
       </c>
       <c r="G28" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H28" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I28" s="34" t="s">
         <v>50</v>
@@ -4837,21 +4848,21 @@
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B29" s="18" t="e">
-        <v>#N/A</v>
+      <c r="B29" s="18" t="s">
+        <v>134</v>
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>103</v>
+        <v>135</v>
       </c>
       <c r="F29" s="32" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="G29" s="33" t="s">
         <v>46</v>
@@ -4864,29 +4875,29 @@
       </c>
       <c r="J29" s="35">
         <f>+IFERROR(VLOOKUP(E29,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
+        <v>44256</v>
       </c>
       <c r="K29" s="45"/>
     </row>
     <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="18" t="e">
+      <c r="A30" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="B30" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B30" s="18" t="s">
-        <v>134</v>
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E30" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="F30" s="32" t="s">
-        <v>134</v>
+        <v>183</v>
+      </c>
+      <c r="F30" s="34" t="s">
+        <v>182</v>
       </c>
       <c r="G30" s="33" t="s">
         <v>46</v>
@@ -4899,7 +4910,7 @@
       </c>
       <c r="J30" s="35">
         <f>+IFERROR(VLOOKUP(E30,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44256</v>
+        <v>44993</v>
       </c>
       <c r="K30" s="45"/>
     </row>
@@ -4912,7 +4923,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4947,7 +4958,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -4974,72 +4985,72 @@
       <c r="K32" s="45"/>
     </row>
     <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="B33" s="18" t="e">
+      <c r="A33" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>43</v>
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D33" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>183</v>
-      </c>
-      <c r="F33" s="34" t="s">
-        <v>182</v>
+        <v>45</v>
+      </c>
+      <c r="F33" s="32" t="s">
+        <v>43</v>
       </c>
       <c r="G33" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I33" s="34" t="s">
         <v>50</v>
       </c>
       <c r="J33" s="35">
         <f>+IFERROR(VLOOKUP(E33,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44993</v>
-      </c>
-      <c r="K33" s="45"/>
+        <v>44118</v>
+      </c>
+      <c r="K33" s="44"/>
     </row>
     <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="F34" s="32" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="G34" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H34" s="33" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="I34" s="34" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="J34" s="35">
         <f>+IFERROR(VLOOKUP(E34,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43672</v>
+        <v>43867</v>
       </c>
       <c r="K34" s="45"/>
     </row>
@@ -5052,7 +5063,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5079,20 +5090,24 @@
       <c r="K35" s="45"/>
     </row>
     <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36"/>
-      <c r="B36"/>
+      <c r="A36" s="18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>78</v>
+      </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
       </c>
       <c r="E36" s="31" t="s">
-        <v>259</v>
+        <v>79</v>
       </c>
       <c r="F36" s="32" t="s">
-        <v>260</v>
+        <v>78</v>
       </c>
       <c r="G36" s="33" t="s">
         <v>46</v>
@@ -5101,68 +5116,68 @@
         <v>47</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="J36" s="35" t="str">
+        <v>50</v>
+      </c>
+      <c r="J36" s="35">
         <f>+IFERROR(VLOOKUP(E36,[1]Sheet1!C:H,6,0),"")</f>
-        <v>29/09/2025</v>
-      </c>
-      <c r="K36" s="47"/>
+        <v>43871</v>
+      </c>
+      <c r="K36" s="45"/>
     </row>
     <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="B37" s="18" t="e">
+      <c r="A37" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>84</v>
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E37" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="F37" s="32" t="s">
-        <v>119</v>
+        <v>44</v>
+      </c>
+      <c r="E37" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="F37" s="39" t="s">
+        <v>84</v>
       </c>
       <c r="G37" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>121</v>
+        <v>50</v>
       </c>
       <c r="J37" s="35">
         <f>+IFERROR(VLOOKUP(E37,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44043</v>
+        <v>43875</v>
       </c>
       <c r="K37" s="45"/>
     </row>
     <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="18" t="e">
-        <v>#N/A</v>
+      <c r="A38" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="B38" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E38" s="31" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="F38" s="32" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="G38" s="33" t="s">
         <v>46</v>
@@ -5175,7 +5190,7 @@
       </c>
       <c r="J38" s="35">
         <f>+IFERROR(VLOOKUP(E38,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44312</v>
+        <v>44043</v>
       </c>
       <c r="K38" s="45"/>
     </row>
@@ -5188,7 +5203,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5218,21 +5233,21 @@
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
-      <c r="B40" s="18" t="s">
-        <v>161</v>
+      <c r="B40" s="18" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E40" s="31" t="s">
-        <v>162</v>
-      </c>
-      <c r="F40" s="32" t="s">
-        <v>161</v>
+      <c r="E40" s="48" t="s">
+        <v>136</v>
+      </c>
+      <c r="F40" s="49" t="s">
+        <v>137</v>
       </c>
       <c r="G40" s="33" t="s">
         <v>46</v>
@@ -5245,7 +5260,7 @@
       </c>
       <c r="J40" s="35">
         <f>+IFERROR(VLOOKUP(E40,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44630</v>
+        <v>44312</v>
       </c>
       <c r="K40" s="45"/>
     </row>
@@ -5254,20 +5269,20 @@
         <v>#N/A</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F41" s="32" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G41" s="33" t="s">
         <v>46</v>
@@ -5280,7 +5295,7 @@
       </c>
       <c r="J41" s="35">
         <f>+IFERROR(VLOOKUP(E41,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44634</v>
+        <v>44630</v>
       </c>
       <c r="K41" s="45"/>
     </row>
@@ -5293,7 +5308,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5328,7 +5343,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5359,20 +5374,20 @@
         <v>#N/A</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E44" s="31" t="s">
-        <v>172</v>
-      </c>
-      <c r="F44" s="34" t="s">
-        <v>171</v>
+        <v>166</v>
+      </c>
+      <c r="F44" s="32" t="s">
+        <v>165</v>
       </c>
       <c r="G44" s="33" t="s">
         <v>46</v>
@@ -5385,7 +5400,7 @@
       </c>
       <c r="J44" s="35">
         <f>+IFERROR(VLOOKUP(E44,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44707</v>
+        <v>44634</v>
       </c>
       <c r="K44" s="45"/>
     </row>
@@ -5394,68 +5409,68 @@
         <v>#N/A</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>48</v>
+        <v>171</v>
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D45" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="E45" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="F45" s="32" t="s">
-        <v>48</v>
+        <v>60</v>
+      </c>
+      <c r="E45" s="48" t="s">
+        <v>172</v>
+      </c>
+      <c r="F45" s="50" t="s">
+        <v>171</v>
       </c>
       <c r="G45" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H45" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I45" s="34" t="s">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="J45" s="35">
         <f>+IFERROR(VLOOKUP(E45,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43040</v>
-      </c>
-      <c r="K45" s="44"/>
+        <v>44707</v>
+      </c>
+      <c r="K45" s="45"/>
     </row>
     <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B46" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D46" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="E46" s="37" t="s">
-        <v>57</v>
+        <v>60</v>
+      </c>
+      <c r="E46" s="31" t="s">
+        <v>68</v>
       </c>
       <c r="F46" s="32" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="G46" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H46" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I46" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J46" s="35">
         <f>+IFERROR(VLOOKUP(E46,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43356</v>
+        <v>43867</v>
       </c>
       <c r="K46" s="45"/>
     </row>
@@ -5468,7 +5483,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5495,37 +5510,37 @@
       <c r="K47" s="45"/>
     </row>
     <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="B48" s="18" t="e">
+      <c r="A48" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>115</v>
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D48" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E48" s="31" t="s">
-        <v>64</v>
+        <v>116</v>
       </c>
       <c r="F48" s="32" t="s">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="G48" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H48" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I48" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J48" s="35">
         <f>+IFERROR(VLOOKUP(E48,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43808</v>
+        <v>44029</v>
       </c>
       <c r="K48" s="45"/>
     </row>
@@ -5538,7 +5553,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5573,7 +5588,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5600,37 +5615,37 @@
       <c r="K50" s="45"/>
     </row>
     <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="18" t="s">
-        <v>65</v>
+      <c r="A51" s="18" t="e">
+        <v>#N/A</v>
       </c>
       <c r="B51" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D51" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="F51" s="32" t="s">
-        <v>65</v>
+        <v>125</v>
       </c>
       <c r="G51" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H51" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I51" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J51" s="35">
         <f>+IFERROR(VLOOKUP(E51,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43803</v>
+        <v>44077</v>
       </c>
       <c r="K51" s="45"/>
     </row>
@@ -5643,7 +5658,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5670,24 +5685,24 @@
       <c r="K52" s="45"/>
     </row>
     <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B53" s="18" t="e">
+      <c r="A53" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>147</v>
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E53" s="31" t="s">
-        <v>68</v>
-      </c>
-      <c r="F53" s="32" t="s">
-        <v>67</v>
+        <v>148</v>
+      </c>
+      <c r="F53" s="39" t="s">
+        <v>147</v>
       </c>
       <c r="G53" s="33" t="s">
         <v>46</v>
@@ -5700,7 +5715,7 @@
       </c>
       <c r="J53" s="35">
         <f>+IFERROR(VLOOKUP(E53,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43867</v>
+        <v>44516</v>
       </c>
       <c r="K53" s="45"/>
     </row>
@@ -5713,7 +5728,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5744,33 +5759,33 @@
         <v>#N/A</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>82</v>
+        <v>155</v>
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="E55" s="38" t="s">
-        <v>83</v>
-      </c>
-      <c r="F55" s="39" t="s">
-        <v>82</v>
+        <v>60</v>
+      </c>
+      <c r="E55" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="F55" s="32" t="s">
+        <v>155</v>
       </c>
       <c r="G55" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H55" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I55" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J55" s="35">
         <f>+IFERROR(VLOOKUP(E55,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
+        <v>44603</v>
       </c>
       <c r="K55" s="45"/>
     </row>
@@ -5783,7 +5798,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5810,37 +5825,37 @@
       <c r="K56" s="45"/>
     </row>
     <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="18" t="e">
+      <c r="A57" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B57" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B57" s="18" t="s">
-        <v>95</v>
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="F57" s="32" t="s">
-        <v>95</v>
+        <v>157</v>
       </c>
       <c r="G57" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H57" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I57" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J57" s="35">
         <f>+IFERROR(VLOOKUP(E57,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43846</v>
+        <v>44610</v>
       </c>
       <c r="K57" s="45"/>
     </row>
@@ -5853,7 +5868,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5888,7 +5903,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5915,59 +5930,55 @@
       <c r="K59" s="45"/>
     </row>
     <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="18" t="e">
+      <c r="A60" s="18" t="s">
+        <v>200</v>
+      </c>
+      <c r="B60" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B60" s="18" t="s">
-        <v>101</v>
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D60" s="30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="E60" s="31" t="s">
-        <v>102</v>
+        <v>201</v>
       </c>
       <c r="F60" s="32" t="s">
-        <v>101</v>
+        <v>200</v>
       </c>
       <c r="G60" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H60" s="33" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="I60" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J60" s="35">
         <f>+IFERROR(VLOOKUP(E60,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43867</v>
-      </c>
-      <c r="K60" s="45"/>
-    </row>
-    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="B61" s="18" t="e">
-        <v>#N/A</v>
-      </c>
+        <v>45372</v>
+      </c>
+      <c r="K60" s="46"/>
+    </row>
+    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61"/>
+      <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E61" s="38" t="s">
-        <v>106</v>
-      </c>
-      <c r="F61" s="39" t="s">
-        <v>105</v>
+      <c r="E61" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="F61" s="32" t="s">
+        <v>260</v>
       </c>
       <c r="G61" s="33" t="s">
         <v>46</v>
@@ -5976,13 +5987,13 @@
         <v>47</v>
       </c>
       <c r="I61" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="J61" s="35">
+        <v>94</v>
+      </c>
+      <c r="J61" s="35" t="str">
         <f>+IFERROR(VLOOKUP(E61,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43875</v>
-      </c>
-      <c r="K61" s="45"/>
+        <v>29/09/2025</v>
+      </c>
+      <c r="K61" s="47"/>
     </row>
     <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="18" t="s">
@@ -5993,7 +6004,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6028,7 +6039,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6063,7 +6074,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6098,7 +6109,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6129,20 +6140,20 @@
         <v>#N/A</v>
       </c>
       <c r="B66" s="18" t="s">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
       </c>
       <c r="E66" s="37" t="s">
-        <v>110</v>
+        <v>49</v>
       </c>
       <c r="F66" s="32" t="s">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="G66" s="33" t="s">
         <v>46</v>
@@ -6155,9 +6166,9 @@
       </c>
       <c r="J66" s="35">
         <f>+IFERROR(VLOOKUP(E66,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43844</v>
-      </c>
-      <c r="K66" s="45"/>
+        <v>43040</v>
+      </c>
+      <c r="K66" s="44"/>
     </row>
     <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="18" t="e">
@@ -6168,7 +6179,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6203,7 +6214,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6238,7 +6249,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6265,94 +6276,94 @@
       <c r="K69" s="45"/>
     </row>
     <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="18" t="e">
+      <c r="A70" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B70" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B70" s="18" t="s">
-        <v>115</v>
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E70" s="31" t="s">
-        <v>116</v>
+        <v>44</v>
+      </c>
+      <c r="E70" s="37" t="s">
+        <v>57</v>
       </c>
       <c r="F70" s="32" t="s">
-        <v>115</v>
+        <v>56</v>
       </c>
       <c r="G70" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H70" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I70" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J70" s="35">
         <f>+IFERROR(VLOOKUP(E70,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44029</v>
+        <v>43356</v>
       </c>
       <c r="K70" s="45"/>
     </row>
     <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="18" t="e">
-        <v>#N/A</v>
+      <c r="A71" s="18" t="s">
+        <v>63</v>
       </c>
       <c r="B71" s="18" t="e">
         <v>#N/A</v>
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D71" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E71" s="31" t="s">
-        <v>124</v>
+        <v>64</v>
       </c>
       <c r="F71" s="32" t="s">
-        <v>125</v>
+        <v>63</v>
       </c>
       <c r="G71" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H71" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I71" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J71" s="35">
         <f>+IFERROR(VLOOKUP(E71,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44077</v>
+        <v>43808</v>
       </c>
       <c r="K71" s="45"/>
     </row>
     <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="18" t="e">
+      <c r="A72" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B72" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B72" s="18" t="s">
-        <v>128</v>
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
       </c>
       <c r="E72" s="31" t="s">
-        <v>129</v>
+        <v>66</v>
       </c>
       <c r="F72" s="32" t="s">
-        <v>128</v>
+        <v>65</v>
       </c>
       <c r="G72" s="33" t="s">
         <v>46</v>
@@ -6365,7 +6376,7 @@
       </c>
       <c r="J72" s="35">
         <f>+IFERROR(VLOOKUP(E72,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44118</v>
+        <v>43803</v>
       </c>
       <c r="K72" s="45"/>
     </row>
@@ -6374,33 +6385,33 @@
         <v>#N/A</v>
       </c>
       <c r="B73" s="18" t="s">
-        <v>147</v>
+        <v>82</v>
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D73" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E73" s="31" t="s">
-        <v>148</v>
+        <v>44</v>
+      </c>
+      <c r="E73" s="38" t="s">
+        <v>83</v>
       </c>
       <c r="F73" s="39" t="s">
-        <v>147</v>
+        <v>82</v>
       </c>
       <c r="G73" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H73" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I73" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J73" s="35">
         <f>+IFERROR(VLOOKUP(E73,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44516</v>
+        <v>43875</v>
       </c>
       <c r="K73" s="45"/>
     </row>
@@ -6409,68 +6420,68 @@
         <v>#N/A</v>
       </c>
       <c r="B74" s="18" t="s">
-        <v>155</v>
+        <v>95</v>
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D74" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E74" s="31" t="s">
-        <v>156</v>
+        <v>96</v>
       </c>
       <c r="F74" s="32" t="s">
-        <v>155</v>
+        <v>95</v>
       </c>
       <c r="G74" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H74" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I74" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J74" s="35">
         <f>+IFERROR(VLOOKUP(E74,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44603</v>
+        <v>43846</v>
       </c>
       <c r="K74" s="45"/>
     </row>
     <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="B75" s="18" t="e">
+      <c r="A75" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B75" s="18" t="s">
+        <v>101</v>
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D75" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E75" s="31" t="s">
-        <v>158</v>
+        <v>102</v>
       </c>
       <c r="F75" s="32" t="s">
-        <v>157</v>
+        <v>101</v>
       </c>
       <c r="G75" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H75" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I75" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J75" s="35">
         <f>+IFERROR(VLOOKUP(E75,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44610</v>
+        <v>43867</v>
       </c>
       <c r="K75" s="45"/>
     </row>
@@ -6483,7 +6494,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6518,7 +6529,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6545,24 +6556,24 @@
       <c r="K77" s="45"/>
     </row>
     <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="18" t="e">
+      <c r="A78" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B78" s="18" t="s">
-        <v>159</v>
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E78" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="F78" s="32" t="s">
-        <v>159</v>
+      <c r="E78" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="F78" s="39" t="s">
+        <v>105</v>
       </c>
       <c r="G78" s="33" t="s">
         <v>46</v>
@@ -6575,7 +6586,7 @@
       </c>
       <c r="J78" s="35">
         <f>+IFERROR(VLOOKUP(E78,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44630</v>
+        <v>43875</v>
       </c>
       <c r="K78" s="45"/>
     </row>
@@ -6588,7 +6599,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6623,7 +6634,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6658,7 +6669,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6693,7 +6704,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6720,24 +6731,24 @@
       <c r="K82" s="45"/>
     </row>
     <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="B83" s="18" t="e">
+      <c r="A83" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B83" s="18" t="s">
+        <v>109</v>
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E83" s="31" t="s">
-        <v>164</v>
+      <c r="E83" s="37" t="s">
+        <v>110</v>
       </c>
       <c r="F83" s="32" t="s">
-        <v>163</v>
+        <v>109</v>
       </c>
       <c r="G83" s="33" t="s">
         <v>46</v>
@@ -6750,7 +6761,7 @@
       </c>
       <c r="J83" s="35">
         <f>+IFERROR(VLOOKUP(E83,[1]Sheet1!C:H,6,0),"")</f>
-        <v>44634</v>
+        <v>43844</v>
       </c>
       <c r="K83" s="45"/>
     </row>
@@ -6763,7 +6774,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6798,7 +6809,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6833,7 +6844,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6868,7 +6879,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6903,7 +6914,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6938,7 +6949,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -6973,7 +6984,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7000,39 +7011,39 @@
       <c r="K90" s="46"/>
     </row>
     <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="B91" s="18" t="e">
+      <c r="A91" s="18" t="e">
         <v>#N/A</v>
+      </c>
+      <c r="B91" s="18" t="s">
+        <v>128</v>
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D91" s="30" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E91" s="31" t="s">
-        <v>201</v>
+        <v>129</v>
       </c>
       <c r="F91" s="32" t="s">
-        <v>200</v>
+        <v>128</v>
       </c>
       <c r="G91" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H91" s="33" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="I91" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J91" s="35">
         <f>+IFERROR(VLOOKUP(E91,[1]Sheet1!C:H,6,0),"")</f>
-        <v>45372</v>
-      </c>
-      <c r="K91" s="46"/>
+        <v>44118</v>
+      </c>
+      <c r="K91" s="45"/>
     </row>
     <row r="92" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="18" t="e">
@@ -7043,7 +7054,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7078,7 +7089,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7113,7 +7124,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7148,7 +7159,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7177,7 +7188,7 @@
     <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7203,10 +7214,10 @@
       </c>
       <c r="K96" s="46"/>
     </row>
-    <row r="97" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7232,10 +7243,10 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7261,10 +7272,10 @@
       </c>
       <c r="K98" s="46"/>
     </row>
-    <row r="99" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7290,10 +7301,10 @@
       </c>
       <c r="K99" s="46"/>
     </row>
-    <row r="100" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7321,10 +7332,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="101" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7350,39 +7361,45 @@
       </c>
       <c r="K101" s="47"/>
     </row>
-    <row r="102" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="B102" s="18" t="s">
+        <v>159</v>
+      </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D102" s="30" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E102" s="31" t="s">
-        <v>222</v>
+        <v>160</v>
       </c>
       <c r="F102" s="32" t="s">
-        <v>223</v>
+        <v>159</v>
       </c>
       <c r="G102" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H102" s="33" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="I102" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="J102" s="35" t="str">
+        <v>58</v>
+      </c>
+      <c r="J102" s="35">
         <f>+IFERROR(VLOOKUP(E102,[1]Sheet1!C:H,6,0),"")</f>
-        <v>30/09/2024</v>
-      </c>
-      <c r="K102" s="47"/>
-    </row>
-    <row r="103" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>44630</v>
+      </c>
+      <c r="K102" s="45"/>
+    </row>
+    <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7408,10 +7425,10 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7437,10 +7454,10 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="3:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7466,10 +7483,10 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7495,10 +7512,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7524,10 +7541,10 @@
       </c>
       <c r="K107" s="47"/>
     </row>
-    <row r="108" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7553,10 +7570,10 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7582,10 +7599,10 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7611,10 +7628,10 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7640,10 +7657,10 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7672,7 +7689,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7701,7 +7718,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7730,7 +7747,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7759,7 +7776,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7788,7 +7805,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7817,7 +7834,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7844,44 +7861,44 @@
       <c r="K118" s="47"/>
     </row>
     <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="18" t="e">
+      <c r="A119" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="B119" s="18" t="e">
         <v>#N/A</v>
-      </c>
-      <c r="B119" s="18" t="s">
-        <v>86</v>
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D119" s="30" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E119" s="31" t="s">
-        <v>87</v>
+        <v>164</v>
       </c>
       <c r="F119" s="32" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="G119" s="33" t="s">
         <v>46</v>
       </c>
       <c r="H119" s="33" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="I119" s="34" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="J119" s="35">
         <f>+IFERROR(VLOOKUP(E119,[1]Sheet1!C:H,6,0),"")</f>
-        <v>43903</v>
+        <v>44634</v>
       </c>
       <c r="K119" s="45"/>
     </row>
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7910,7 +7927,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7938,7 +7955,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -7966,7 +7983,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -7994,7 +8011,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8022,7 +8039,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8050,7 +8067,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8078,7 +8095,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8106,7 +8123,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8134,7 +8151,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8162,7 +8179,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8190,7 +8207,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8218,7 +8235,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8246,7 +8263,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8274,7 +8291,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8304,7 +8321,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8332,7 +8349,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8360,7 +8377,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8388,7 +8405,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8416,7 +8433,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8444,7 +8461,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8475,7 +8492,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8506,7 +8523,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8538,15 +8555,12 @@
   <autoFilter ref="A21:FL142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
     <filterColumn colId="8">
       <filters>
-        <filter val="Group Leader"/>
-        <filter val="Junior Technician"/>
         <filter val="Operator"/>
         <filter val="Skilled worker"/>
-        <filter val="Supervisor"/>
         <filter val="Team Leader"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A22:K119">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A27:K119">
       <sortCondition descending="1" ref="I21:I142"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
Final sync and push to Vercel
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFCFBBC9-FCD5-4844-B74F-B34C4805BF99}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E5E59E7-5D69-4F59-B113-0D1A104E4AB6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -33,7 +33,7 @@
     <definedName name="_4M画面移動_.メニュー画面">#REF!</definedName>
     <definedName name="_50票製造部区分3___a">#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tháng 04.2026'!$A$21:$FL$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tháng 04.2026'!$A$21:$K$142</definedName>
     <definedName name="_Key1" hidden="1">#REF!</definedName>
     <definedName name="_M18">#REF!</definedName>
     <definedName name="_Order1" hidden="1">0</definedName>
@@ -1723,7 +1723,26 @@
     <cellStyle name="Normal 4" xfId="4" xr:uid="{65BE7283-C593-425E-BBF3-D3B7608B399D}"/>
     <cellStyle name="一般_Sheet1" xfId="3" xr:uid="{FE885AC6-95BF-4FD1-A89B-BE2A4049A73C}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -4775,7 +4794,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4809,7 +4828,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4818,7 +4837,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4844,7 +4863,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4853,7 +4872,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4879,7 +4898,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="18" t="s">
         <v>182</v>
       </c>
@@ -4888,7 +4907,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4923,7 +4942,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4958,7 +4977,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -4984,7 +5003,7 @@
       </c>
       <c r="K32" s="45"/>
     </row>
-    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4993,7 +5012,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5019,7 +5038,7 @@
       </c>
       <c r="K33" s="44"/>
     </row>
-    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5028,7 +5047,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5063,7 +5082,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5089,7 +5108,7 @@
       </c>
       <c r="K35" s="45"/>
     </row>
-    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5098,7 +5117,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5124,7 +5143,7 @@
       </c>
       <c r="K36" s="45"/>
     </row>
-    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5133,7 +5152,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5159,7 +5178,7 @@
       </c>
       <c r="K37" s="45"/>
     </row>
-    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="18" t="s">
         <v>119</v>
       </c>
@@ -5168,7 +5187,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5203,7 +5222,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5229,7 +5248,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5238,7 +5257,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5264,7 +5283,7 @@
       </c>
       <c r="K40" s="45"/>
     </row>
-    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5273,7 +5292,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5308,7 +5327,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5343,7 +5362,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5369,7 +5388,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5378,7 +5397,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5404,7 +5423,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5413,7 +5432,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5439,7 +5458,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
         <v>67</v>
       </c>
@@ -5448,7 +5467,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5483,7 +5502,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5509,7 +5528,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5518,7 +5537,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5553,7 +5572,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5588,7 +5607,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5614,7 +5633,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5623,7 +5642,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5658,7 +5677,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5684,7 +5703,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5693,7 +5712,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5719,7 +5738,7 @@
       </c>
       <c r="K53" s="45"/>
     </row>
-    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5728,7 +5747,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5746,7 +5765,7 @@
         <v>47</v>
       </c>
       <c r="I54" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J54" s="35">
         <f>+IFERROR(VLOOKUP(E54,[1]Sheet1!C:H,6,0),"")</f>
@@ -5754,7 +5773,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5763,7 +5782,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5798,7 +5817,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5824,7 +5843,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="18" t="s">
         <v>157</v>
       </c>
@@ -5833,7 +5852,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5868,7 +5887,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5903,7 +5922,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5929,7 +5948,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="18" t="s">
         <v>200</v>
       </c>
@@ -5938,7 +5957,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5969,7 +5988,7 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6004,7 +6023,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6039,7 +6058,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6074,7 +6093,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6109,7 +6128,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6135,7 +6154,7 @@
       </c>
       <c r="K65" s="45"/>
     </row>
-    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6144,7 +6163,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6179,7 +6198,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6214,7 +6233,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6249,7 +6268,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6284,7 +6303,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6319,7 +6338,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6354,7 +6373,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6389,7 +6408,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6424,7 +6443,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6459,7 +6478,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6494,7 +6513,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6529,7 +6548,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6564,7 +6583,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6599,7 +6618,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6634,7 +6653,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6669,7 +6688,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6704,7 +6723,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6730,7 +6749,7 @@
       </c>
       <c r="K82" s="45"/>
     </row>
-    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6739,7 +6758,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6774,7 +6793,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6809,7 +6828,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6844,7 +6863,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6879,7 +6898,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6914,7 +6933,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6940,7 +6959,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6949,7 +6968,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -6967,7 +6986,7 @@
         <v>47</v>
       </c>
       <c r="I89" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J89" s="35">
         <f>+IFERROR(VLOOKUP(E89,[1]Sheet1!C:H,6,0),"")</f>
@@ -6975,7 +6994,7 @@
       </c>
       <c r="K89" s="46"/>
     </row>
-    <row r="90" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6984,7 +7003,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7002,7 +7021,7 @@
         <v>47</v>
       </c>
       <c r="I90" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J90" s="35">
         <f>+IFERROR(VLOOKUP(E90,[1]Sheet1!C:H,6,0),"")</f>
@@ -7019,7 +7038,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7054,7 +7073,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7089,7 +7108,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7124,7 +7143,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7150,7 +7169,7 @@
       </c>
       <c r="K94" s="46"/>
     </row>
-    <row r="95" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7159,7 +7178,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7177,7 +7196,7 @@
         <v>47</v>
       </c>
       <c r="I95" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J95" s="35">
         <f>+IFERROR(VLOOKUP(E95,[1]Sheet1!C:H,6,0),"")</f>
@@ -7185,10 +7204,10 @@
       </c>
       <c r="K95" s="46"/>
     </row>
-    <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7206,7 +7225,7 @@
         <v>47</v>
       </c>
       <c r="I96" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J96" s="35">
         <f>+IFERROR(VLOOKUP(E96,[1]Sheet1!C:H,6,0),"")</f>
@@ -7217,7 +7236,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7243,10 +7262,10 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7264,7 +7283,7 @@
         <v>47</v>
       </c>
       <c r="I98" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J98" s="35" t="str">
         <f>+IFERROR(VLOOKUP(E98,[1]Sheet1!C:H,6,0),"")</f>
@@ -7275,7 +7294,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7304,7 +7323,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7335,7 +7354,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7370,7 +7389,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7396,10 +7415,10 @@
       </c>
       <c r="K102" s="45"/>
     </row>
-    <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7417,7 +7436,7 @@
         <v>47</v>
       </c>
       <c r="I103" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J103" s="35" t="str">
         <f>+IFERROR(VLOOKUP(E103,[1]Sheet1!C:H,6,0),"")</f>
@@ -7428,7 +7447,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7457,7 +7476,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7483,10 +7502,10 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7504,7 +7523,7 @@
         <v>47</v>
       </c>
       <c r="I106" s="34" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J106" s="35" t="str">
         <f>+IFERROR(VLOOKUP(E106,[1]Sheet1!C:H,6,0),"")</f>
@@ -7515,7 +7534,7 @@
     <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7544,7 +7563,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7573,7 +7592,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7602,7 +7621,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7631,7 +7650,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7660,7 +7679,7 @@
     <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7689,7 +7708,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7718,7 +7737,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7747,7 +7766,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7776,7 +7795,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7805,7 +7824,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7834,7 +7853,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7869,7 +7888,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7898,7 +7917,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7927,7 +7946,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7955,7 +7974,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -7983,7 +8002,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8011,7 +8030,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8039,7 +8058,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8067,7 +8086,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8095,7 +8114,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8123,7 +8142,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8151,7 +8170,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8179,7 +8198,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8207,7 +8226,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8235,7 +8254,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8263,7 +8282,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8291,7 +8310,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8321,7 +8340,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8349,7 +8368,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8377,7 +8396,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8405,7 +8424,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8433,7 +8452,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8461,7 +8480,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8492,7 +8511,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8523,7 +8542,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8552,18 +8571,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A21:FL142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="Operator"/>
-        <filter val="Skilled worker"/>
-        <filter val="Team Leader"/>
-      </filters>
+  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
+    <filterColumn colId="4">
+      <colorFilter dxfId="0"/>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A27:K119">
-      <sortCondition descending="1" ref="I21:I142"/>
-    </sortState>
   </autoFilter>
+  <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>

<commit_message>
Add operator dropdown filters based on department and position
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E5E59E7-5D69-4F59-B113-0D1A104E4AB6}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42ED22C3-448C-45BE-A1CE-5E62E9A38E8F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -1723,15 +1723,7 @@
     <cellStyle name="Normal 4" xfId="4" xr:uid="{65BE7283-C593-425E-BBF3-D3B7608B399D}"/>
     <cellStyle name="一般_Sheet1" xfId="3" xr:uid="{FE885AC6-95BF-4FD1-A89B-BE2A4049A73C}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4794,7 +4786,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4828,7 +4820,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4837,7 +4829,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4863,7 +4855,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4872,7 +4864,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4898,7 +4890,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="18" t="s">
         <v>182</v>
       </c>
@@ -4907,7 +4899,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4942,7 +4934,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4977,7 +4969,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5003,7 +4995,7 @@
       </c>
       <c r="K32" s="45"/>
     </row>
-    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5012,7 +5004,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5038,7 +5030,7 @@
       </c>
       <c r="K33" s="44"/>
     </row>
-    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5047,7 +5039,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5082,7 +5074,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5108,7 +5100,7 @@
       </c>
       <c r="K35" s="45"/>
     </row>
-    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5117,7 +5109,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5143,7 +5135,7 @@
       </c>
       <c r="K36" s="45"/>
     </row>
-    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5152,7 +5144,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5187,7 +5179,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5222,7 +5214,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5248,7 +5240,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5257,7 +5249,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5275,7 +5267,7 @@
         <v>62</v>
       </c>
       <c r="I40" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J40" s="35">
         <f>+IFERROR(VLOOKUP(E40,[1]Sheet1!C:H,6,0),"")</f>
@@ -5292,7 +5284,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5327,7 +5319,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5362,7 +5354,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5397,7 +5389,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5423,7 +5415,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5432,7 +5424,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5450,7 +5442,7 @@
         <v>62</v>
       </c>
       <c r="I45" s="34" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="J45" s="35">
         <f>+IFERROR(VLOOKUP(E45,[1]Sheet1!C:H,6,0),"")</f>
@@ -5458,7 +5450,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
         <v>67</v>
       </c>
@@ -5467,7 +5459,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5502,7 +5494,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5528,7 +5520,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5537,7 +5529,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5572,7 +5564,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5607,7 +5599,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5633,7 +5625,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5642,7 +5634,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5677,7 +5669,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5703,7 +5695,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5712,7 +5704,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5747,7 +5739,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5773,7 +5765,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5782,7 +5774,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5817,7 +5809,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5843,7 +5835,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="18" t="s">
         <v>157</v>
       </c>
@@ -5852,7 +5844,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5887,7 +5879,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5922,7 +5914,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5948,7 +5940,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="18" t="s">
         <v>200</v>
       </c>
@@ -5957,7 +5949,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5988,7 +5980,7 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6023,7 +6015,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6058,7 +6050,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6093,7 +6085,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6128,7 +6120,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6154,7 +6146,7 @@
       </c>
       <c r="K65" s="45"/>
     </row>
-    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6163,7 +6155,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6198,7 +6190,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6233,7 +6225,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6268,7 +6260,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6303,7 +6295,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6338,7 +6330,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6373,7 +6365,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6408,7 +6400,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6443,7 +6435,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6478,7 +6470,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6513,7 +6505,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6548,7 +6540,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6583,7 +6575,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6618,7 +6610,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6653,7 +6645,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6688,7 +6680,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6723,7 +6715,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6749,7 +6741,7 @@
       </c>
       <c r="K82" s="45"/>
     </row>
-    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6758,7 +6750,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6793,7 +6785,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6828,7 +6820,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6863,7 +6855,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6898,7 +6890,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6933,7 +6925,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6968,7 +6960,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -7003,7 +6995,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7038,7 +7030,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7073,7 +7065,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7108,7 +7100,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7143,7 +7135,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7178,7 +7170,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7207,7 +7199,7 @@
     <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7236,7 +7228,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7265,7 +7257,7 @@
     <row r="98" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7294,7 +7286,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7323,7 +7315,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7354,7 +7346,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7389,7 +7381,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7418,7 +7410,7 @@
     <row r="103" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7447,7 +7439,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7476,7 +7468,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7505,7 +7497,7 @@
     <row r="106" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7534,7 +7526,7 @@
     <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7563,7 +7555,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7592,7 +7584,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7621,7 +7613,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7650,7 +7642,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7679,7 +7671,7 @@
     <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7708,7 +7700,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7737,7 +7729,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7766,7 +7758,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7795,7 +7787,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7824,7 +7816,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7853,7 +7845,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7888,7 +7880,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7917,7 +7909,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7946,7 +7938,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7974,7 +7966,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -8002,7 +7994,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8030,7 +8022,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8058,7 +8050,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8086,7 +8078,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8114,7 +8106,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8142,7 +8134,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8170,7 +8162,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8198,7 +8190,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8226,7 +8218,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8254,7 +8246,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8282,7 +8274,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8310,7 +8302,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8340,7 +8332,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8368,7 +8360,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8396,7 +8388,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8424,7 +8416,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8452,7 +8444,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8480,7 +8472,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8511,7 +8503,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8542,7 +8534,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8572,12 +8564,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-    <filterColumn colId="4">
-      <colorFilter dxfId="0"/>
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Operator"/>
+        <filter val="Team Leader"/>
+      </filters>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: them loi soc dao, mm khong deu, mong day vao danh sach loi may tach
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42ED22C3-448C-45BE-A1CE-5E62E9A38E8F}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E036063E-D1D4-4791-A25A-60B4C4CFD892}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4820,7 +4820,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4855,7 +4855,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="18" t="s">
         <v>182</v>
       </c>
@@ -4899,7 +4899,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4969,7 +4969,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5389,7 +5389,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="s">
         <v>67</v>
       </c>
@@ -5459,7 +5459,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5625,7 +5625,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5634,7 +5634,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5765,7 +5765,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5809,7 +5809,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5835,7 +5835,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="18" t="s">
         <v>157</v>
       </c>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="18" t="s">
         <v>200</v>
       </c>
@@ -5949,7 +5949,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5980,7 +5980,7 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6050,7 +6050,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6085,7 +6085,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6260,7 +6260,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6505,7 +6505,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6680,7 +6680,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6715,7 +6715,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6925,7 +6925,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7100,7 +7100,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7135,7 +7135,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7199,7 +7199,7 @@
     <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7228,7 +7228,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7257,7 +7257,7 @@
     <row r="98" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7286,7 +7286,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7315,7 +7315,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7346,7 +7346,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7381,7 +7381,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7410,7 +7410,7 @@
     <row r="103" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7439,7 +7439,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7468,7 +7468,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7497,7 +7497,7 @@
     <row r="106" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7526,7 +7526,7 @@
     <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7555,7 +7555,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7584,7 +7584,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7613,7 +7613,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7642,7 +7642,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7671,7 +7671,7 @@
     <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7700,7 +7700,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7729,7 +7729,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7758,7 +7758,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7787,7 +7787,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7816,7 +7816,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7845,7 +7845,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7909,7 +7909,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7938,7 +7938,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7966,7 +7966,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -7994,7 +7994,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8022,7 +8022,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8050,7 +8050,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8078,7 +8078,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8106,7 +8106,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8134,7 +8134,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8162,7 +8162,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8190,7 +8190,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8218,7 +8218,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8246,7 +8246,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8274,7 +8274,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8302,7 +8302,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8332,7 +8332,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8360,7 +8360,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8388,7 +8388,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8416,7 +8416,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8444,7 +8444,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8472,7 +8472,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8503,7 +8503,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8534,7 +8534,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8564,6 +8564,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="FOAMING Splitting"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="8">
       <filters>
         <filter val="Operator"/>

</xml_diff>

<commit_message>
feat: cap nhat do day bun tham chieu mac dinh 144mm khi chua co tieu chuan
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{915D4DC6-EECB-4F11-9A8A-EA77DC514E23}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8AB31B7-5A78-4FB0-8F9B-B5154E995643}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -4339,7 +4339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:K142"/>
@@ -4654,12 +4654,12 @@
       </c>
       <c r="K22" s="45"/>
     </row>
-    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23" s="29">
         <f>IF(E23&lt;&gt;"",SUBTOTAL(103,E$22:E23),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="30" t="s">
         <v>72</v>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="K23" s="47"/>
     </row>
-    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="C24" s="29">
         <f>IF(E24&lt;&gt;"",SUBTOTAL(103,E$22:E24),"")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>44</v>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="K24" s="44"/>
     </row>
-    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="C25" s="29">
         <f>IF(E25&lt;&gt;"",SUBTOTAL(103,E$22:E25),"")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>44</v>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="K25" s="44"/>
     </row>
-    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C26" s="29">
         <f>IF(E26&lt;&gt;"",SUBTOTAL(103,E$22:E26),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D26" s="30" t="s">
         <v>72</v>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="K30" s="45"/>
     </row>
-    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="K31" s="45"/>
     </row>
-    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4973,7 +4973,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="K34" s="45"/>
     </row>
-    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5113,7 +5113,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="K37" s="45"/>
     </row>
-    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="18" t="s">
         <v>119</v>
       </c>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5209,7 +5209,7 @@
       </c>
       <c r="K38" s="45"/>
     </row>
-    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="K40" s="45"/>
     </row>
-    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="K42" s="45"/>
     </row>
-    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="18" t="s">
         <v>67</v>
       </c>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="K46" s="45"/>
     </row>
-    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="K48" s="45"/>
     </row>
-    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="18" t="s">
         <v>111</v>
       </c>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="K49" s="45"/>
     </row>
-    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5664,7 +5664,7 @@
       </c>
       <c r="K51" s="45"/>
     </row>
-    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5734,7 +5734,7 @@
       </c>
       <c r="K53" s="45"/>
     </row>
-    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5743,7 +5743,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="K55" s="45"/>
     </row>
-    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5839,7 +5839,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="18" t="s">
         <v>157</v>
       </c>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5874,7 +5874,7 @@
       </c>
       <c r="K57" s="45"/>
     </row>
-    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5909,7 +5909,7 @@
       </c>
       <c r="K58" s="45"/>
     </row>
-    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="18" t="s">
         <v>200</v>
       </c>
@@ -5953,7 +5953,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5984,7 +5984,7 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6010,7 +6010,7 @@
       </c>
       <c r="K61" s="47"/>
     </row>
-    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="18" t="s">
         <v>138</v>
       </c>
@@ -6019,7 +6019,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="K62" s="45"/>
     </row>
-    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6054,7 +6054,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="K63" s="45"/>
     </row>
-    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6115,7 +6115,7 @@
       </c>
       <c r="K64" s="45"/>
     </row>
-    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="18" t="s">
         <v>145</v>
       </c>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="K65" s="45"/>
     </row>
-    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6159,7 +6159,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6185,7 +6185,7 @@
       </c>
       <c r="K66" s="44"/>
     </row>
-    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6194,7 +6194,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="K67" s="45"/>
     </row>
-    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="18" t="s">
         <v>151</v>
       </c>
@@ -6229,7 +6229,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="K68" s="45"/>
     </row>
-    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6290,7 +6290,7 @@
       </c>
       <c r="K69" s="45"/>
     </row>
-    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="18" t="s">
         <v>56</v>
       </c>
@@ -6299,7 +6299,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6325,7 +6325,7 @@
       </c>
       <c r="K70" s="45"/>
     </row>
-    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="18" t="s">
         <v>63</v>
       </c>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6360,7 +6360,7 @@
       </c>
       <c r="K71" s="45"/>
     </row>
-    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="18" t="s">
         <v>65</v>
       </c>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="K72" s="45"/>
     </row>
-    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="K73" s="45"/>
     </row>
-    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6439,7 +6439,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="K74" s="45"/>
     </row>
-    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6500,7 +6500,7 @@
       </c>
       <c r="K75" s="45"/>
     </row>
-    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="18" t="s">
         <v>167</v>
       </c>
@@ -6509,7 +6509,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6535,7 +6535,7 @@
       </c>
       <c r="K76" s="45"/>
     </row>
-    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6570,7 +6570,7 @@
       </c>
       <c r="K77" s="45"/>
     </row>
-    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="18" t="s">
         <v>105</v>
       </c>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6640,7 +6640,7 @@
       </c>
       <c r="K79" s="45"/>
     </row>
-    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="K80" s="45"/>
     </row>
-    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6710,7 +6710,7 @@
       </c>
       <c r="K81" s="45"/>
     </row>
-    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6745,7 +6745,7 @@
       </c>
       <c r="K82" s="45"/>
     </row>
-    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="K83" s="45"/>
     </row>
-    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6789,7 +6789,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6815,7 +6815,7 @@
       </c>
       <c r="K84" s="45"/>
     </row>
-    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6850,7 +6850,7 @@
       </c>
       <c r="K85" s="45"/>
     </row>
-    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6859,7 +6859,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="K86" s="45"/>
     </row>
-    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6894,7 +6894,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6920,7 +6920,7 @@
       </c>
       <c r="K87" s="45"/>
     </row>
-    <row r="88" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="18" t="s">
         <v>194</v>
       </c>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6955,7 +6955,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="K89" s="46"/>
     </row>
-    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7025,7 +7025,7 @@
       </c>
       <c r="K90" s="46"/>
     </row>
-    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7060,7 +7060,7 @@
       </c>
       <c r="K91" s="45"/>
     </row>
-    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="K92" s="46"/>
     </row>
-    <row r="93" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="18" t="s">
         <v>204</v>
       </c>
@@ -7104,7 +7104,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7130,7 +7130,7 @@
       </c>
       <c r="K93" s="46"/>
     </row>
-    <row r="94" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7139,7 +7139,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>73</v>
+        <v>10</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7165,7 +7165,7 @@
       </c>
       <c r="K94" s="46"/>
     </row>
-    <row r="95" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7200,10 +7200,10 @@
       </c>
       <c r="K95" s="46"/>
     </row>
-    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7229,10 +7229,10 @@
       </c>
       <c r="K96" s="46"/>
     </row>
-    <row r="97" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7258,10 +7258,10 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7287,10 +7287,10 @@
       </c>
       <c r="K98" s="46"/>
     </row>
-    <row r="99" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7316,10 +7316,10 @@
       </c>
       <c r="K99" s="46"/>
     </row>
-    <row r="100" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7347,10 +7347,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="101" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="K101" s="47"/>
     </row>
-    <row r="102" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7385,7 +7385,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7411,10 +7411,10 @@
       </c>
       <c r="K102" s="45"/>
     </row>
-    <row r="103" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7440,10 +7440,10 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>83</v>
+        <v>10</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7469,10 +7469,10 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>84</v>
+        <v>10</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7498,10 +7498,10 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7527,10 +7527,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7556,10 +7556,10 @@
       </c>
       <c r="K107" s="47"/>
     </row>
-    <row r="108" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7585,10 +7585,10 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>88</v>
+        <v>10</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7614,10 +7614,10 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7643,10 +7643,10 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7672,10 +7672,10 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7701,10 +7701,10 @@
       </c>
       <c r="K112" s="47"/>
     </row>
-    <row r="113" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7730,10 +7730,10 @@
       </c>
       <c r="K113" s="47"/>
     </row>
-    <row r="114" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7759,10 +7759,10 @@
       </c>
       <c r="K114" s="47"/>
     </row>
-    <row r="115" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7788,10 +7788,10 @@
       </c>
       <c r="K115" s="47"/>
     </row>
-    <row r="116" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7817,10 +7817,10 @@
       </c>
       <c r="K116" s="47"/>
     </row>
-    <row r="117" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7846,10 +7846,10 @@
       </c>
       <c r="K117" s="47"/>
     </row>
-    <row r="118" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7875,7 +7875,7 @@
       </c>
       <c r="K118" s="47"/>
     </row>
-    <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="18" t="s">
         <v>163</v>
       </c>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7910,10 +7910,10 @@
       </c>
       <c r="K119" s="45"/>
     </row>
-    <row r="120" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7939,10 +7939,10 @@
       </c>
       <c r="K120" s="47"/>
     </row>
-    <row r="121" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7967,10 +7967,10 @@
       </c>
       <c r="K121" s="47"/>
     </row>
-    <row r="122" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>101</v>
+        <v>10</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -7995,10 +7995,10 @@
       </c>
       <c r="K122" s="47"/>
     </row>
-    <row r="123" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8023,10 +8023,10 @@
       </c>
       <c r="K123" s="47"/>
     </row>
-    <row r="124" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>103</v>
+        <v>10</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8051,10 +8051,10 @@
       </c>
       <c r="K124" s="47"/>
     </row>
-    <row r="125" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8079,10 +8079,10 @@
       </c>
       <c r="K125" s="47"/>
     </row>
-    <row r="126" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8107,10 +8107,10 @@
       </c>
       <c r="K126" s="47"/>
     </row>
-    <row r="127" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>106</v>
+        <v>10</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8135,10 +8135,10 @@
       </c>
       <c r="K127" s="47"/>
     </row>
-    <row r="128" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8163,10 +8163,10 @@
       </c>
       <c r="K128" s="47"/>
     </row>
-    <row r="129" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>108</v>
+        <v>10</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8191,10 +8191,10 @@
       </c>
       <c r="K129" s="47"/>
     </row>
-    <row r="130" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>109</v>
+        <v>10</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8219,10 +8219,10 @@
       </c>
       <c r="K130" s="47"/>
     </row>
-    <row r="131" spans="3:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>110</v>
+        <v>10</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8247,10 +8247,10 @@
       </c>
       <c r="K131" s="47"/>
     </row>
-    <row r="132" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>111</v>
+        <v>10</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8275,10 +8275,10 @@
       </c>
       <c r="K132" s="47"/>
     </row>
-    <row r="133" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>112</v>
+        <v>10</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8303,10 +8303,10 @@
       </c>
       <c r="K133" s="47"/>
     </row>
-    <row r="134" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>113</v>
+        <v>10</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8333,10 +8333,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>114</v>
+        <v>10</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8361,10 +8361,10 @@
       </c>
       <c r="K135" s="46"/>
     </row>
-    <row r="136" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>115</v>
+        <v>10</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8389,10 +8389,10 @@
       </c>
       <c r="K136" s="46"/>
     </row>
-    <row r="137" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>116</v>
+        <v>10</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8417,10 +8417,10 @@
       </c>
       <c r="K137" s="46"/>
     </row>
-    <row r="138" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8445,10 +8445,10 @@
       </c>
       <c r="K138" s="46"/>
     </row>
-    <row r="139" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>118</v>
+        <v>10</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8473,10 +8473,10 @@
       </c>
       <c r="K139" s="46"/>
     </row>
-    <row r="140" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>119</v>
+        <v>10</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8504,10 +8504,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="141" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8535,10 +8535,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="142" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>121</v>
+        <v>10</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8567,7 +8567,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}"/>
+  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Supervisor"/>
+        <filter val="Team Leader"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: add is_compensation (Don bu) option for pour and separate reports, update production plan sheets
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8AB31B7-5A78-4FB0-8F9B-B5154E995643}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AC6B8CE-A547-44F4-A4A4-C5E1302D6756}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="319">
   <si>
     <t>D</t>
   </si>
@@ -1339,6 +1339,15 @@
   </si>
   <si>
     <t>Đã nghỉ việc đang tuyển thay thế</t>
+  </si>
+  <si>
+    <t>Dương Vĩnh Lâm</t>
+  </si>
+  <si>
+    <t>Foaming Supervisor</t>
+  </si>
+  <si>
+    <t>18/7/2024</t>
   </si>
 </sst>
 </file>
@@ -1571,7 +1580,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1712,7 +1721,16 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1723,7 +1741,15 @@
     <cellStyle name="Normal 4" xfId="4" xr:uid="{65BE7283-C593-425E-BBF3-D3B7608B399D}"/>
     <cellStyle name="一般_Sheet1" xfId="3" xr:uid="{FE885AC6-95BF-4FD1-A89B-BE2A4049A73C}"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4036,10 +4062,6 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4342,7 +4364,7 @@
   <sheetPr filterMode="1">
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:K142"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.6328125" hidden="1" customWidth="1"/>
@@ -4619,7 +4641,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4628,7 +4650,7 @@
       </c>
       <c r="C22" s="29">
         <f>IF(E22&lt;&gt;"",SUBTOTAL(103,E$22:E22),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="30" t="s">
         <v>72</v>
@@ -4659,7 +4681,7 @@
       <c r="B23"/>
       <c r="C23" s="29">
         <f>IF(E23&lt;&gt;"",SUBTOTAL(103,E$22:E23),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" s="30" t="s">
         <v>72</v>
@@ -4694,7 +4716,7 @@
       </c>
       <c r="C24" s="29">
         <f>IF(E24&lt;&gt;"",SUBTOTAL(103,E$22:E24),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>44</v>
@@ -4729,7 +4751,7 @@
       </c>
       <c r="C25" s="29">
         <f>IF(E25&lt;&gt;"",SUBTOTAL(103,E$22:E25),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>44</v>
@@ -4764,7 +4786,7 @@
       </c>
       <c r="C26" s="29">
         <f>IF(E26&lt;&gt;"",SUBTOTAL(103,E$22:E26),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" s="30" t="s">
         <v>72</v>
@@ -4803,10 +4825,10 @@
       <c r="D27" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="31" t="s">
+      <c r="E27" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="F27" s="32" t="s">
+      <c r="F27" s="49" t="s">
         <v>59</v>
       </c>
       <c r="G27" s="33" t="s">
@@ -4824,7 +4846,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4833,7 +4855,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4859,7 +4881,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4868,7 +4890,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4894,7 +4916,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="18" t="s">
         <v>182</v>
       </c>
@@ -4903,7 +4925,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4938,7 +4960,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4973,7 +4995,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5008,15 +5030,15 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E33" s="31" t="s">
+      <c r="E33" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="F33" s="32" t="s">
+      <c r="F33" s="49" t="s">
         <v>43</v>
       </c>
       <c r="G33" s="33" t="s">
@@ -5034,7 +5056,7 @@
       </c>
       <c r="K33" s="44"/>
     </row>
-    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5043,7 +5065,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5078,7 +5100,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5104,7 +5126,7 @@
       </c>
       <c r="K35" s="45"/>
     </row>
-    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5113,7 +5135,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5139,7 +5161,7 @@
       </c>
       <c r="K36" s="45"/>
     </row>
-    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5148,7 +5170,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5183,7 +5205,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5218,7 +5240,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5253,15 +5275,15 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E40" s="48" t="s">
+      <c r="E40" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="F40" s="49" t="s">
+      <c r="F40" s="52" t="s">
         <v>137</v>
       </c>
       <c r="G40" s="33" t="s">
@@ -5288,7 +5310,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5323,7 +5345,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5358,7 +5380,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5393,7 +5415,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5428,15 +5450,15 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E45" s="48" t="s">
+      <c r="E45" s="51" t="s">
         <v>172</v>
       </c>
-      <c r="F45" s="50" t="s">
+      <c r="F45" s="53" t="s">
         <v>171</v>
       </c>
       <c r="G45" s="33" t="s">
@@ -5463,7 +5485,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5498,7 +5520,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5533,7 +5555,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5568,7 +5590,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5603,7 +5625,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5638,7 +5660,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5673,7 +5695,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5708,7 +5730,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5743,7 +5765,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5778,7 +5800,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5813,7 +5835,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5848,7 +5870,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5883,7 +5905,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5918,7 +5940,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5953,7 +5975,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5984,15 +6006,15 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E61" s="31" t="s">
+      <c r="E61" s="48" t="s">
         <v>259</v>
       </c>
-      <c r="F61" s="32" t="s">
+      <c r="F61" s="49" t="s">
         <v>260</v>
       </c>
       <c r="G61" s="33" t="s">
@@ -6019,7 +6041,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6054,7 +6076,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6089,7 +6111,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6124,7 +6146,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6159,7 +6181,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6194,7 +6216,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6229,7 +6251,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6264,7 +6286,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6299,7 +6321,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6334,7 +6356,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6369,7 +6391,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6404,7 +6426,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6439,7 +6461,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6474,7 +6496,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6509,7 +6531,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6544,7 +6566,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6579,7 +6601,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6614,7 +6636,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6649,7 +6671,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6684,7 +6706,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6719,7 +6741,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6754,7 +6776,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6789,7 +6811,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6824,7 +6846,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6859,7 +6881,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6894,7 +6916,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6929,7 +6951,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6964,7 +6986,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -6999,7 +7021,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7034,7 +7056,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7069,7 +7091,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7104,7 +7126,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7139,7 +7161,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7174,7 +7196,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7203,7 +7225,7 @@
     <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7232,7 +7254,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7261,7 +7283,7 @@
     <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7290,7 +7312,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7319,7 +7341,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7350,7 +7372,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7385,7 +7407,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7414,7 +7436,7 @@
     <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7443,7 +7465,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7472,7 +7494,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7501,7 +7523,7 @@
     <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7530,7 +7552,7 @@
     <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7559,7 +7581,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7588,7 +7610,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7617,7 +7639,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7646,7 +7668,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7675,7 +7697,7 @@
     <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7704,7 +7726,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7733,7 +7755,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7762,7 +7784,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7791,7 +7813,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7820,7 +7842,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7849,7 +7871,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7884,7 +7906,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7913,7 +7935,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7942,7 +7964,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7970,7 +7992,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -7998,7 +8020,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8026,7 +8048,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8054,7 +8076,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8082,7 +8104,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8110,7 +8132,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8138,7 +8160,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8166,7 +8188,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8194,7 +8216,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8222,7 +8244,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8250,7 +8272,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8278,7 +8300,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8306,7 +8328,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8336,7 +8358,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8364,7 +8386,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8392,7 +8414,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8420,7 +8442,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8448,7 +8470,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8476,7 +8498,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8507,7 +8529,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8538,7 +8560,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8566,17 +8588,41 @@
         <v>310</v>
       </c>
     </row>
+    <row r="143" spans="3:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C143" s="42">
+        <v>122</v>
+      </c>
+      <c r="D143" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="E143" s="50">
+        <v>4127</v>
+      </c>
+      <c r="F143" s="49" t="s">
+        <v>316</v>
+      </c>
+      <c r="G143" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="H143" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="I143" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="J143" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="K143" s="47"/>
+    </row>
   </sheetData>
   <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="Supervisor"/>
-        <filter val="Team Leader"/>
-      </filters>
+    <filterColumn colId="5">
+      <colorFilter dxfId="0"/>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Update weekly production plans and foaming progress for W23-2026
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AC6B8CE-A547-44F4-A4A4-C5E1302D6756}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9810913-E7C1-43E8-BA61-DE7F1F62F86B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -1580,7 +1580,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1724,15 +1724,6 @@
     <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1741,15 +1732,7 @@
     <cellStyle name="Normal 4" xfId="4" xr:uid="{65BE7283-C593-425E-BBF3-D3B7608B399D}"/>
     <cellStyle name="一般_Sheet1" xfId="3" xr:uid="{FE885AC6-95BF-4FD1-A89B-BE2A4049A73C}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4812,7 +4795,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4855,7 +4838,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4890,7 +4873,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4925,7 +4908,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4960,7 +4943,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4995,7 +4978,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5021,7 +5004,7 @@
       </c>
       <c r="K32" s="45"/>
     </row>
-    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5030,7 +5013,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5065,7 +5048,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5100,7 +5083,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5135,7 +5118,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5170,7 +5153,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5205,7 +5188,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5240,7 +5223,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5275,15 +5258,15 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E40" s="51" t="s">
+      <c r="E40" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="F40" s="52" t="s">
+      <c r="F40" s="32" t="s">
         <v>137</v>
       </c>
       <c r="G40" s="33" t="s">
@@ -5310,7 +5293,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5336,7 +5319,7 @@
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5345,7 +5328,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5380,7 +5363,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5406,7 +5389,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5455,10 +5438,10 @@
       <c r="D45" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E45" s="51" t="s">
+      <c r="E45" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="F45" s="53" t="s">
+      <c r="F45" s="34" t="s">
         <v>171</v>
       </c>
       <c r="G45" s="33" t="s">
@@ -6001,12 +5984,12 @@
       </c>
       <c r="K60" s="46"/>
     </row>
-    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61"/>
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6041,7 +6024,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6076,7 +6059,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6111,7 +6094,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6146,7 +6129,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6181,7 +6164,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6216,7 +6199,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6251,7 +6234,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6286,7 +6269,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6321,7 +6304,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6356,7 +6339,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6391,7 +6374,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6426,7 +6409,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6461,7 +6444,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6496,7 +6479,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6531,7 +6514,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6566,7 +6549,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6601,7 +6584,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6627,7 +6610,7 @@
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6977,7 +6960,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6986,7 +6969,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -7021,7 +7004,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7056,7 +7039,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7091,7 +7074,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7126,7 +7109,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7161,7 +7144,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7196,7 +7179,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7225,7 +7208,7 @@
     <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7254,7 +7237,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7283,7 +7266,7 @@
     <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7312,7 +7295,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7341,7 +7324,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7372,7 +7355,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7407,7 +7390,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7436,7 +7419,7 @@
     <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7465,7 +7448,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7494,7 +7477,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7523,7 +7506,7 @@
     <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7549,10 +7532,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7581,7 +7564,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7610,7 +7593,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7639,7 +7622,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7668,7 +7651,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7697,7 +7680,7 @@
     <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7726,7 +7709,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7755,7 +7738,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7784,7 +7767,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7813,7 +7796,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7842,7 +7825,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7871,7 +7854,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7906,7 +7889,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7935,7 +7918,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7964,7 +7947,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7992,7 +7975,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -8020,7 +8003,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8048,7 +8031,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8076,7 +8059,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8104,7 +8087,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8132,7 +8115,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8160,7 +8143,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8188,7 +8171,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8216,7 +8199,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8244,7 +8227,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8272,7 +8255,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8300,7 +8283,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8328,7 +8311,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8358,7 +8341,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8386,7 +8369,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8414,7 +8397,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8442,7 +8425,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8470,7 +8453,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8498,7 +8481,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8529,7 +8512,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8560,7 +8543,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8618,11 +8601,17 @@
   </sheetData>
   <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
     <filterColumn colId="5">
-      <colorFilter dxfId="0"/>
+      <filters>
+        <filter val="Lê Đoàn Vũ"/>
+        <filter val="Ngô Vũ Luân"/>
+        <filter val="Ngô Vũ Phương"/>
+        <filter val="Nguyễn Tuấn Vũ"/>
+        <filter val="Nguyễn Vũ Em"/>
+      </filters>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
data: update foaming list and sample production plan Excel files
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9810913-E7C1-43E8-BA61-DE7F1F62F86B}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8106C8A1-D269-4B33-BA3C-3A6C373BC1B3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5389,7 +5389,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5398,7 +5398,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5468,7 +5468,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5503,7 +5503,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5713,7 +5713,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5853,7 +5853,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5989,7 +5989,7 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6024,7 +6024,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6059,7 +6059,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D63" s="30" t="s">
         <v>72</v>
@@ -6094,7 +6094,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6234,7 +6234,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6269,7 +6269,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6304,7 +6304,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6374,7 +6374,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6409,7 +6409,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6619,7 +6619,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6689,7 +6689,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6759,7 +6759,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6829,7 +6829,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6899,7 +6899,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6934,7 +6934,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6969,7 +6969,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7039,7 +7039,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7144,7 +7144,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7208,7 +7208,7 @@
     <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7237,7 +7237,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7266,7 +7266,7 @@
     <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7295,7 +7295,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7324,7 +7324,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7355,7 +7355,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7390,7 +7390,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7419,7 +7419,7 @@
     <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7448,7 +7448,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7477,7 +7477,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7506,7 +7506,7 @@
     <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7532,10 +7532,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7564,7 +7564,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7593,7 +7593,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7622,7 +7622,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7651,7 +7651,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7677,10 +7677,10 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7709,7 +7709,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7738,7 +7738,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7767,7 +7767,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7796,7 +7796,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7825,7 +7825,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7854,7 +7854,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7918,7 +7918,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7947,7 +7947,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7975,7 +7975,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -8003,7 +8003,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8031,7 +8031,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8059,7 +8059,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8087,7 +8087,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8115,7 +8115,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8143,7 +8143,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8171,7 +8171,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8199,7 +8199,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8227,7 +8227,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8255,7 +8255,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8283,7 +8283,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8311,7 +8311,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8341,7 +8341,7 @@
     <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8369,7 +8369,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8397,7 +8397,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8425,7 +8425,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8453,7 +8453,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8481,7 +8481,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8512,7 +8512,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8543,7 +8543,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8602,11 +8602,7 @@
   <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
     <filterColumn colId="5">
       <filters>
-        <filter val="Lê Đoàn Vũ"/>
-        <filter val="Ngô Vũ Luân"/>
-        <filter val="Ngô Vũ Phương"/>
-        <filter val="Nguyễn Tuấn Vũ"/>
-        <filter val="Nguyễn Vũ Em"/>
+        <filter val="Danh Tiền"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
data: cap nhat du lieu sample moi nhat sheet 8.6
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8106C8A1-D269-4B33-BA3C-3A6C373BC1B3}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E4947ED-1171-4B57-8CBE-6868E3161315}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -1580,7 +1580,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1724,6 +1724,9 @@
     <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="7" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1732,7 +1735,15 @@
     <cellStyle name="Normal 4" xfId="4" xr:uid="{65BE7283-C593-425E-BBF3-D3B7608B399D}"/>
     <cellStyle name="一般_Sheet1" xfId="3" xr:uid="{FE885AC6-95BF-4FD1-A89B-BE2A4049A73C}"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4795,7 +4806,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4838,7 +4849,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4873,7 +4884,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4908,7 +4919,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4943,7 +4954,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4978,7 +4989,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5004,7 +5015,7 @@
       </c>
       <c r="K32" s="45"/>
     </row>
-    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5013,7 +5024,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5048,7 +5059,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5083,7 +5094,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5118,7 +5129,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5153,7 +5164,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5188,7 +5199,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5223,7 +5234,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5258,7 +5269,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5293,7 +5304,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5328,7 +5339,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5363,7 +5374,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5398,7 +5409,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5433,7 +5444,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5468,7 +5479,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5503,7 +5514,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5538,7 +5549,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5573,7 +5584,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5608,7 +5619,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5643,7 +5654,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5678,7 +5689,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5713,7 +5724,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5748,7 +5759,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5783,7 +5794,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5818,7 +5829,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5853,7 +5864,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5888,7 +5899,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5923,7 +5934,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5958,7 +5969,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -5984,12 +5995,12 @@
       </c>
       <c r="K60" s="46"/>
     </row>
-    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61"/>
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6024,7 +6035,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6050,7 +6061,7 @@
       </c>
       <c r="K62" s="45"/>
     </row>
-    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6059,15 +6070,15 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>0</v>
-      </c>
-      <c r="D63" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="D63" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="E63" s="31" t="s">
+      <c r="E63" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="F63" s="32" t="s">
+      <c r="F63" s="49" t="s">
         <v>140</v>
       </c>
       <c r="G63" s="33" t="s">
@@ -6094,7 +6105,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6129,7 +6140,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6164,7 +6175,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6199,7 +6210,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6234,7 +6245,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6269,7 +6280,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6304,7 +6315,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6339,7 +6350,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6374,7 +6385,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6409,7 +6420,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6444,7 +6455,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6479,7 +6490,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6514,7 +6525,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6549,7 +6560,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6584,7 +6595,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6619,7 +6630,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6654,7 +6665,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6689,7 +6700,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6724,7 +6735,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6759,7 +6770,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6794,7 +6805,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6829,7 +6840,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6864,7 +6875,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6890,7 +6901,7 @@
       </c>
       <c r="K86" s="45"/>
     </row>
-    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6899,15 +6910,15 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E87" s="31" t="s">
+      <c r="E87" s="48" t="s">
         <v>192</v>
       </c>
-      <c r="F87" s="32" t="s">
+      <c r="F87" s="49" t="s">
         <v>191</v>
       </c>
       <c r="G87" s="33" t="s">
@@ -6934,7 +6945,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6969,7 +6980,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -7004,7 +7015,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7039,7 +7050,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7074,7 +7085,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7109,7 +7120,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7144,7 +7155,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7179,7 +7190,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7208,7 +7219,7 @@
     <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7237,7 +7248,7 @@
     <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7266,7 +7277,7 @@
     <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7295,7 +7306,7 @@
     <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7324,7 +7335,7 @@
     <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7355,7 +7366,7 @@
     <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7390,7 +7401,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7419,7 +7430,7 @@
     <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7448,7 +7459,7 @@
     <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7477,7 +7488,7 @@
     <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7506,7 +7517,7 @@
     <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7535,7 +7546,7 @@
     <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7564,7 +7575,7 @@
     <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7593,7 +7604,7 @@
     <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7622,7 +7633,7 @@
     <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7651,7 +7662,7 @@
     <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7677,10 +7688,10 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7709,7 +7720,7 @@
     <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7738,7 +7749,7 @@
     <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7767,7 +7778,7 @@
     <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7796,7 +7807,7 @@
     <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7825,7 +7836,7 @@
     <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7854,7 +7865,7 @@
     <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7889,7 +7900,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7918,7 +7929,7 @@
     <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7947,7 +7958,7 @@
     <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7975,7 +7986,7 @@
     <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -8003,7 +8014,7 @@
     <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8031,7 +8042,7 @@
     <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8059,7 +8070,7 @@
     <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8087,7 +8098,7 @@
     <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8115,7 +8126,7 @@
     <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8143,7 +8154,7 @@
     <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8171,7 +8182,7 @@
     <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8199,7 +8210,7 @@
     <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8227,7 +8238,7 @@
     <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8255,7 +8266,7 @@
     <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8283,7 +8294,7 @@
     <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8311,7 +8322,7 @@
     <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8338,18 +8349,18 @@
         <v>315</v>
       </c>
     </row>
-    <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E135" s="31" t="s">
+      <c r="E135" s="48" t="s">
         <v>295</v>
       </c>
-      <c r="F135" s="32" t="s">
+      <c r="F135" s="49" t="s">
         <v>296</v>
       </c>
       <c r="G135" s="33" t="s">
@@ -8369,7 +8380,7 @@
     <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8397,7 +8408,7 @@
     <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8425,7 +8436,7 @@
     <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8453,7 +8464,7 @@
     <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8481,7 +8492,7 @@
     <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8512,7 +8523,7 @@
     <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8543,7 +8554,7 @@
     <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8601,13 +8612,11 @@
   </sheetData>
   <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
     <filterColumn colId="5">
-      <filters>
-        <filter val="Danh Tiền"/>
-      </filters>
+      <colorFilter dxfId="0"/>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Excel data files
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E4947ED-1171-4B57-8CBE-6868E3161315}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82456587-1E62-494D-99C7-C20719421AF8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -1491,7 +1491,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1519,6 +1519,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1580,7 +1592,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1727,6 +1739,12 @@
     <xf numFmtId="2" fontId="7" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1735,15 +1753,7 @@
     <cellStyle name="Normal 4" xfId="4" xr:uid="{65BE7283-C593-425E-BBF3-D3B7608B399D}"/>
     <cellStyle name="一般_Sheet1" xfId="3" xr:uid="{FE885AC6-95BF-4FD1-A89B-BE2A4049A73C}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4355,7 +4365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:K143"/>
@@ -4635,7 +4645,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4644,7 +4654,7 @@
       </c>
       <c r="C22" s="29">
         <f>IF(E22&lt;&gt;"",SUBTOTAL(103,E$22:E22),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="30" t="s">
         <v>72</v>
@@ -4670,12 +4680,12 @@
       </c>
       <c r="K22" s="45"/>
     </row>
-    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23" s="29">
         <f>IF(E23&lt;&gt;"",SUBTOTAL(103,E$22:E23),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D23" s="30" t="s">
         <v>72</v>
@@ -4701,7 +4711,7 @@
       </c>
       <c r="K23" s="47"/>
     </row>
-    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4710,7 +4720,7 @@
       </c>
       <c r="C24" s="29">
         <f>IF(E24&lt;&gt;"",SUBTOTAL(103,E$22:E24),"")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>44</v>
@@ -4736,7 +4746,7 @@
       </c>
       <c r="K24" s="44"/>
     </row>
-    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4745,7 +4755,7 @@
       </c>
       <c r="C25" s="29">
         <f>IF(E25&lt;&gt;"",SUBTOTAL(103,E$22:E25),"")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>44</v>
@@ -4771,7 +4781,7 @@
       </c>
       <c r="K25" s="44"/>
     </row>
-    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4780,7 +4790,7 @@
       </c>
       <c r="C26" s="29">
         <f>IF(E26&lt;&gt;"",SUBTOTAL(103,E$22:E26),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D26" s="30" t="s">
         <v>72</v>
@@ -4840,7 +4850,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4849,7 +4859,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4875,7 +4885,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4884,7 +4894,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4910,7 +4920,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="18" t="s">
         <v>182</v>
       </c>
@@ -4919,7 +4929,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4945,7 +4955,7 @@
       </c>
       <c r="K30" s="45"/>
     </row>
-    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4954,7 +4964,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4980,7 +4990,7 @@
       </c>
       <c r="K31" s="45"/>
     </row>
-    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4989,7 +4999,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5024,7 +5034,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5050,7 +5060,7 @@
       </c>
       <c r="K33" s="44"/>
     </row>
-    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5059,7 +5069,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5085,7 +5095,7 @@
       </c>
       <c r="K34" s="45"/>
     </row>
-    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5094,7 +5104,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5120,7 +5130,7 @@
       </c>
       <c r="K35" s="45"/>
     </row>
-    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5129,7 +5139,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5155,7 +5165,7 @@
       </c>
       <c r="K36" s="45"/>
     </row>
-    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5164,7 +5174,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5190,7 +5200,7 @@
       </c>
       <c r="K37" s="45"/>
     </row>
-    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="18" t="s">
         <v>119</v>
       </c>
@@ -5199,7 +5209,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5225,7 +5235,7 @@
       </c>
       <c r="K38" s="45"/>
     </row>
-    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5234,7 +5244,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5242,7 +5252,7 @@
       <c r="E39" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="F39" s="32" t="s">
+      <c r="F39" s="52" t="s">
         <v>89</v>
       </c>
       <c r="G39" s="33" t="s">
@@ -5260,7 +5270,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5269,7 +5279,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5295,7 +5305,7 @@
       </c>
       <c r="K40" s="45"/>
     </row>
-    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5304,7 +5314,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5330,7 +5340,7 @@
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5339,7 +5349,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5365,7 +5375,7 @@
       </c>
       <c r="K42" s="45"/>
     </row>
-    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5374,7 +5384,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5400,7 +5410,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5409,7 +5419,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5435,7 +5445,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5444,7 +5454,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5470,7 +5480,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="18" t="s">
         <v>67</v>
       </c>
@@ -5479,7 +5489,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5505,7 +5515,7 @@
       </c>
       <c r="K46" s="45"/>
     </row>
-    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5514,7 +5524,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5540,7 +5550,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5549,7 +5559,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5575,7 +5585,7 @@
       </c>
       <c r="K48" s="45"/>
     </row>
-    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="18" t="s">
         <v>111</v>
       </c>
@@ -5584,7 +5594,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5610,7 +5620,7 @@
       </c>
       <c r="K49" s="45"/>
     </row>
-    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5619,7 +5629,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5627,7 +5637,7 @@
       <c r="E50" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="F50" s="32" t="s">
+      <c r="F50" s="52" t="s">
         <v>113</v>
       </c>
       <c r="G50" s="33" t="s">
@@ -5645,7 +5655,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5654,7 +5664,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5680,7 +5690,7 @@
       </c>
       <c r="K51" s="45"/>
     </row>
-    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5689,7 +5699,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5697,7 +5707,7 @@
       <c r="E52" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="F52" s="32" t="s">
+      <c r="F52" s="53" t="s">
         <v>117</v>
       </c>
       <c r="G52" s="33" t="s">
@@ -5715,7 +5725,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5724,7 +5734,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5750,7 +5760,7 @@
       </c>
       <c r="K53" s="45"/>
     </row>
-    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5759,7 +5769,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5785,7 +5795,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5794,7 +5804,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5820,7 +5830,7 @@
       </c>
       <c r="K55" s="45"/>
     </row>
-    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5829,7 +5839,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5855,7 +5865,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="18" t="s">
         <v>157</v>
       </c>
@@ -5864,7 +5874,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5890,7 +5900,7 @@
       </c>
       <c r="K57" s="45"/>
     </row>
-    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5899,7 +5909,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5925,7 +5935,7 @@
       </c>
       <c r="K58" s="45"/>
     </row>
-    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5934,7 +5944,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5942,7 +5952,7 @@
       <c r="E59" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="F59" s="32" t="s">
+      <c r="F59" s="52" t="s">
         <v>132</v>
       </c>
       <c r="G59" s="33" t="s">
@@ -5960,7 +5970,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="18" t="s">
         <v>200</v>
       </c>
@@ -5969,7 +5979,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -6000,7 +6010,7 @@
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6026,7 +6036,7 @@
       </c>
       <c r="K61" s="47"/>
     </row>
-    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="18" t="s">
         <v>138</v>
       </c>
@@ -6035,7 +6045,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6070,7 +6080,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="D63" s="51" t="s">
         <v>72</v>
@@ -6096,7 +6106,7 @@
       </c>
       <c r="K63" s="45"/>
     </row>
-    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6105,7 +6115,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6131,7 +6141,7 @@
       </c>
       <c r="K64" s="45"/>
     </row>
-    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="18" t="s">
         <v>145</v>
       </c>
@@ -6140,7 +6150,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6166,7 +6176,7 @@
       </c>
       <c r="K65" s="45"/>
     </row>
-    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6175,7 +6185,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6201,7 +6211,7 @@
       </c>
       <c r="K66" s="44"/>
     </row>
-    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6210,7 +6220,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6236,7 +6246,7 @@
       </c>
       <c r="K67" s="45"/>
     </row>
-    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="18" t="s">
         <v>151</v>
       </c>
@@ -6245,7 +6255,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6271,7 +6281,7 @@
       </c>
       <c r="K68" s="45"/>
     </row>
-    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6280,7 +6290,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6288,7 +6298,7 @@
       <c r="E69" s="31" t="s">
         <v>154</v>
       </c>
-      <c r="F69" s="32" t="s">
+      <c r="F69" s="49" t="s">
         <v>153</v>
       </c>
       <c r="G69" s="33" t="s">
@@ -6306,7 +6316,7 @@
       </c>
       <c r="K69" s="45"/>
     </row>
-    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="18" t="s">
         <v>56</v>
       </c>
@@ -6315,7 +6325,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6341,7 +6351,7 @@
       </c>
       <c r="K70" s="45"/>
     </row>
-    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="18" t="s">
         <v>63</v>
       </c>
@@ -6350,7 +6360,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6376,7 +6386,7 @@
       </c>
       <c r="K71" s="45"/>
     </row>
-    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="18" t="s">
         <v>65</v>
       </c>
@@ -6385,7 +6395,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6411,7 +6421,7 @@
       </c>
       <c r="K72" s="45"/>
     </row>
-    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6420,7 +6430,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6446,7 +6456,7 @@
       </c>
       <c r="K73" s="45"/>
     </row>
-    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6455,7 +6465,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6481,7 +6491,7 @@
       </c>
       <c r="K74" s="45"/>
     </row>
-    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6490,7 +6500,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6516,7 +6526,7 @@
       </c>
       <c r="K75" s="45"/>
     </row>
-    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="18" t="s">
         <v>167</v>
       </c>
@@ -6525,7 +6535,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6533,7 +6543,7 @@
       <c r="E76" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="F76" s="32" t="s">
+      <c r="F76" s="52" t="s">
         <v>167</v>
       </c>
       <c r="G76" s="33" t="s">
@@ -6551,7 +6561,7 @@
       </c>
       <c r="K76" s="45"/>
     </row>
-    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6560,7 +6570,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6586,7 +6596,7 @@
       </c>
       <c r="K77" s="45"/>
     </row>
-    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="18" t="s">
         <v>105</v>
       </c>
@@ -6595,7 +6605,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6621,7 +6631,7 @@
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6630,7 +6640,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6656,7 +6666,7 @@
       </c>
       <c r="K79" s="45"/>
     </row>
-    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6665,7 +6675,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6691,7 +6701,7 @@
       </c>
       <c r="K80" s="45"/>
     </row>
-    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6700,7 +6710,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6726,7 +6736,7 @@
       </c>
       <c r="K81" s="45"/>
     </row>
-    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6735,7 +6745,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6761,7 +6771,7 @@
       </c>
       <c r="K82" s="45"/>
     </row>
-    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6770,7 +6780,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6796,7 +6806,7 @@
       </c>
       <c r="K83" s="45"/>
     </row>
-    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6805,7 +6815,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6831,7 +6841,7 @@
       </c>
       <c r="K84" s="45"/>
     </row>
-    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6840,7 +6850,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6866,7 +6876,7 @@
       </c>
       <c r="K85" s="45"/>
     </row>
-    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6875,7 +6885,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6910,7 +6920,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6936,7 +6946,7 @@
       </c>
       <c r="K87" s="45"/>
     </row>
-    <row r="88" spans="1:11" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="18" t="s">
         <v>194</v>
       </c>
@@ -6945,7 +6955,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6971,7 +6981,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6980,7 +6990,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -7006,7 +7016,7 @@
       </c>
       <c r="K89" s="46"/>
     </row>
-    <row r="90" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7015,7 +7025,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>5</v>
+        <v>69</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7041,7 +7051,7 @@
       </c>
       <c r="K90" s="46"/>
     </row>
-    <row r="91" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7050,7 +7060,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7076,7 +7086,7 @@
       </c>
       <c r="K91" s="45"/>
     </row>
-    <row r="92" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7085,7 +7095,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>5</v>
+        <v>71</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7111,7 +7121,7 @@
       </c>
       <c r="K92" s="46"/>
     </row>
-    <row r="93" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="18" t="s">
         <v>204</v>
       </c>
@@ -7120,7 +7130,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7146,7 +7156,7 @@
       </c>
       <c r="K93" s="46"/>
     </row>
-    <row r="94" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7155,7 +7165,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7181,7 +7191,7 @@
       </c>
       <c r="K94" s="46"/>
     </row>
-    <row r="95" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7190,7 +7200,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>5</v>
+        <v>74</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7216,10 +7226,10 @@
       </c>
       <c r="K95" s="46"/>
     </row>
-    <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7245,10 +7255,10 @@
       </c>
       <c r="K96" s="46"/>
     </row>
-    <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>5</v>
+        <v>76</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7274,10 +7284,10 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7303,10 +7313,10 @@
       </c>
       <c r="K98" s="46"/>
     </row>
-    <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>5</v>
+        <v>78</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7332,10 +7342,10 @@
       </c>
       <c r="K99" s="46"/>
     </row>
-    <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>5</v>
+        <v>79</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7363,10 +7373,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7392,7 +7402,7 @@
       </c>
       <c r="K101" s="47"/>
     </row>
-    <row r="102" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7401,7 +7411,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>5</v>
+        <v>81</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7427,10 +7437,10 @@
       </c>
       <c r="K102" s="45"/>
     </row>
-    <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>5</v>
+        <v>82</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7456,10 +7466,10 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7485,10 +7495,10 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7514,10 +7524,10 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7543,10 +7553,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>5</v>
+        <v>86</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7572,10 +7582,10 @@
       </c>
       <c r="K107" s="47"/>
     </row>
-    <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>5</v>
+        <v>87</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7583,7 +7593,7 @@
       <c r="E108" s="31" t="s">
         <v>235</v>
       </c>
-      <c r="F108" s="32" t="s">
+      <c r="F108" s="49" t="s">
         <v>236</v>
       </c>
       <c r="G108" s="33" t="s">
@@ -7601,10 +7611,10 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>5</v>
+        <v>88</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7630,10 +7640,10 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>5</v>
+        <v>89</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7659,10 +7669,10 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7688,10 +7698,10 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>5</v>
+        <v>91</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7717,10 +7727,10 @@
       </c>
       <c r="K112" s="47"/>
     </row>
-    <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>5</v>
+        <v>92</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7746,10 +7756,10 @@
       </c>
       <c r="K113" s="47"/>
     </row>
-    <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>5</v>
+        <v>93</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7775,10 +7785,10 @@
       </c>
       <c r="K114" s="47"/>
     </row>
-    <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7804,10 +7814,10 @@
       </c>
       <c r="K115" s="47"/>
     </row>
-    <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7833,10 +7843,10 @@
       </c>
       <c r="K116" s="47"/>
     </row>
-    <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7862,10 +7872,10 @@
       </c>
       <c r="K117" s="47"/>
     </row>
-    <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7891,7 +7901,7 @@
       </c>
       <c r="K118" s="47"/>
     </row>
-    <row r="119" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="18" t="s">
         <v>163</v>
       </c>
@@ -7900,7 +7910,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>5</v>
+        <v>98</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7926,10 +7936,10 @@
       </c>
       <c r="K119" s="45"/>
     </row>
-    <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7955,10 +7965,10 @@
       </c>
       <c r="K120" s="47"/>
     </row>
-    <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7983,10 +7993,10 @@
       </c>
       <c r="K121" s="47"/>
     </row>
-    <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>5</v>
+        <v>101</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -8011,10 +8021,10 @@
       </c>
       <c r="K122" s="47"/>
     </row>
-    <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8039,10 +8049,10 @@
       </c>
       <c r="K123" s="47"/>
     </row>
-    <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>5</v>
+        <v>103</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8067,10 +8077,10 @@
       </c>
       <c r="K124" s="47"/>
     </row>
-    <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>5</v>
+        <v>104</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8095,10 +8105,10 @@
       </c>
       <c r="K125" s="47"/>
     </row>
-    <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>5</v>
+        <v>105</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8123,10 +8133,10 @@
       </c>
       <c r="K126" s="47"/>
     </row>
-    <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>5</v>
+        <v>106</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8151,10 +8161,10 @@
       </c>
       <c r="K127" s="47"/>
     </row>
-    <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>5</v>
+        <v>107</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8179,10 +8189,10 @@
       </c>
       <c r="K128" s="47"/>
     </row>
-    <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>5</v>
+        <v>108</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8207,10 +8217,10 @@
       </c>
       <c r="K129" s="47"/>
     </row>
-    <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>5</v>
+        <v>109</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8235,10 +8245,10 @@
       </c>
       <c r="K130" s="47"/>
     </row>
-    <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>5</v>
+        <v>110</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8263,10 +8273,10 @@
       </c>
       <c r="K131" s="47"/>
     </row>
-    <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>5</v>
+        <v>111</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8291,10 +8301,10 @@
       </c>
       <c r="K132" s="47"/>
     </row>
-    <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>5</v>
+        <v>112</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8319,10 +8329,10 @@
       </c>
       <c r="K133" s="47"/>
     </row>
-    <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>5</v>
+        <v>113</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8352,7 +8362,7 @@
     <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>6</v>
+        <v>114</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8377,10 +8387,10 @@
       </c>
       <c r="K135" s="46"/>
     </row>
-    <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>6</v>
+        <v>115</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8405,10 +8415,10 @@
       </c>
       <c r="K136" s="46"/>
     </row>
-    <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>6</v>
+        <v>116</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8433,10 +8443,10 @@
       </c>
       <c r="K137" s="46"/>
     </row>
-    <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>6</v>
+        <v>117</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8461,10 +8471,10 @@
       </c>
       <c r="K138" s="46"/>
     </row>
-    <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>6</v>
+        <v>118</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8489,10 +8499,10 @@
       </c>
       <c r="K139" s="46"/>
     </row>
-    <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>6</v>
+        <v>119</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8520,10 +8530,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>6</v>
+        <v>120</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8551,10 +8561,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>6</v>
+        <v>121</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8610,13 +8620,9 @@
       <c r="K143" s="47"/>
     </row>
   </sheetData>
-  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-    <filterColumn colId="5">
-      <colorFilter dxfId="0"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}"/>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
data: update foaming and production excel sheets, and add supabase storage columns schema
</commit_message>
<xml_diff>
--- a/DS Hiện tại bộ phận Foaming.xlsx
+++ b/DS Hiện tại bộ phận Foaming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82456587-1E62-494D-99C7-C20719421AF8}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="13_ncr:1_{E7AC9B5B-8808-463F-A1B6-5E43E5806A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19540407-E2F7-4269-8A52-1697682AA3FA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3841106A-7DEB-4CF0-913D-81EEFFBEFE28}"/>
   </bookViews>
@@ -4365,7 +4365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:K143"/>
@@ -4645,7 +4645,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4654,7 +4654,7 @@
       </c>
       <c r="C22" s="29">
         <f>IF(E22&lt;&gt;"",SUBTOTAL(103,E$22:E22),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="30" t="s">
         <v>72</v>
@@ -4680,12 +4680,12 @@
       </c>
       <c r="K22" s="45"/>
     </row>
-    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" s="18" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23" s="29">
         <f>IF(E23&lt;&gt;"",SUBTOTAL(103,E$22:E23),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D23" s="30" t="s">
         <v>72</v>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="K23" s="47"/>
     </row>
-    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="C24" s="29">
         <f>IF(E24&lt;&gt;"",SUBTOTAL(103,E$22:E24),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>44</v>
@@ -4746,7 +4746,7 @@
       </c>
       <c r="K24" s="44"/>
     </row>
-    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" s="18" customFormat="1" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="C25" s="29">
         <f>IF(E25&lt;&gt;"",SUBTOTAL(103,E$22:E25),"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>44</v>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="K25" s="44"/>
     </row>
-    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="C26" s="29">
         <f>IF(E26&lt;&gt;"",SUBTOTAL(103,E$22:E26),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D26" s="30" t="s">
         <v>72</v>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="K26" s="45"/>
     </row>
-    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="18" t="s">
         <v>59</v>
       </c>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="K27" s="45"/>
     </row>
-    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="C28" s="29">
         <f>IF(E28&lt;&gt;"",SUBTOTAL(103,E$22:E28),"")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>60</v>
@@ -4885,7 +4885,7 @@
       </c>
       <c r="K28" s="45"/>
     </row>
-    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="C29" s="29">
         <f>IF(E29&lt;&gt;"",SUBTOTAL(103,E$22:E29),"")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>60</v>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="K29" s="45"/>
     </row>
-    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="18" t="s">
         <v>182</v>
       </c>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="C30" s="29">
         <f>IF(E30&lt;&gt;"",SUBTOTAL(103,E$22:E30),"")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>60</v>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="K30" s="45"/>
     </row>
-    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C31" s="29">
         <f>IF(E31&lt;&gt;"",SUBTOTAL(103,E$22:E31),"")</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>44</v>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="K31" s="45"/>
     </row>
-    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="C32" s="29">
         <f>IF(E32&lt;&gt;"",SUBTOTAL(103,E$22:E32),"")</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>72</v>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="K32" s="45"/>
     </row>
-    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="C33" s="29">
         <f>IF(E33&lt;&gt;"",SUBTOTAL(103,E$22:E33),"")</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>44</v>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="K33" s="44"/>
     </row>
-    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="C34" s="29">
         <f>IF(E34&lt;&gt;"",SUBTOTAL(103,E$22:E34),"")</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D34" s="30" t="s">
         <v>44</v>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="K34" s="45"/>
     </row>
-    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="C35" s="29">
         <f>IF(E35&lt;&gt;"",SUBTOTAL(103,E$22:E35),"")</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>60</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="K35" s="45"/>
     </row>
-    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5139,7 +5139,7 @@
       </c>
       <c r="C36" s="29">
         <f>IF(E36&lt;&gt;"",SUBTOTAL(103,E$22:E36),"")</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>44</v>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="K36" s="45"/>
     </row>
-    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="C37" s="29">
         <f>IF(E37&lt;&gt;"",SUBTOTAL(103,E$22:E37),"")</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>44</v>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="K37" s="45"/>
     </row>
-    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="18" t="s">
         <v>119</v>
       </c>
@@ -5209,7 +5209,7 @@
       </c>
       <c r="C38" s="29">
         <f>IF(E38&lt;&gt;"",SUBTOTAL(103,E$22:E38),"")</f>
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>60</v>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="K38" s="45"/>
     </row>
-    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="C39" s="29">
         <f>IF(E39&lt;&gt;"",SUBTOTAL(103,E$22:E39),"")</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>72</v>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="K39" s="45"/>
     </row>
-    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="C40" s="29">
         <f>IF(E40&lt;&gt;"",SUBTOTAL(103,E$22:E40),"")</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>60</v>
@@ -5305,7 +5305,7 @@
       </c>
       <c r="K40" s="45"/>
     </row>
-    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C41" s="29">
         <f>IF(E41&lt;&gt;"",SUBTOTAL(103,E$22:E41),"")</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>60</v>
@@ -5340,7 +5340,7 @@
       </c>
       <c r="K41" s="45"/>
     </row>
-    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="C42" s="29">
         <f>IF(E42&lt;&gt;"",SUBTOTAL(103,E$22:E42),"")</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>60</v>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="C43" s="29">
         <f>IF(E43&lt;&gt;"",SUBTOTAL(103,E$22:E43),"")</f>
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>60</v>
@@ -5410,7 +5410,7 @@
       </c>
       <c r="K43" s="45"/>
     </row>
-    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C44" s="29">
         <f>IF(E44&lt;&gt;"",SUBTOTAL(103,E$22:E44),"")</f>
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>60</v>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="K44" s="45"/>
     </row>
-    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="C45" s="29">
         <f>IF(E45&lt;&gt;"",SUBTOTAL(103,E$22:E45),"")</f>
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="D45" s="30" t="s">
         <v>60</v>
@@ -5480,7 +5480,7 @@
       </c>
       <c r="K45" s="45"/>
     </row>
-    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="18" t="s">
         <v>67</v>
       </c>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="C46" s="29">
         <f>IF(E46&lt;&gt;"",SUBTOTAL(103,E$22:E46),"")</f>
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>60</v>
@@ -5515,7 +5515,7 @@
       </c>
       <c r="K46" s="45"/>
     </row>
-    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="C47" s="29">
         <f>IF(E47&lt;&gt;"",SUBTOTAL(103,E$22:E47),"")</f>
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>44</v>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="K47" s="45"/>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="C48" s="29">
         <f>IF(E48&lt;&gt;"",SUBTOTAL(103,E$22:E48),"")</f>
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>60</v>
@@ -5585,7 +5585,7 @@
       </c>
       <c r="K48" s="45"/>
     </row>
-    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="18" t="s">
         <v>111</v>
       </c>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="C49" s="29">
         <f>IF(E49&lt;&gt;"",SUBTOTAL(103,E$22:E49),"")</f>
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D49" s="30" t="s">
         <v>44</v>
@@ -5620,7 +5620,7 @@
       </c>
       <c r="K49" s="45"/>
     </row>
-    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="C50" s="29">
         <f>IF(E50&lt;&gt;"",SUBTOTAL(103,E$22:E50),"")</f>
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>44</v>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="K50" s="45"/>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C51" s="29">
         <f>IF(E51&lt;&gt;"",SUBTOTAL(103,E$22:E51),"")</f>
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>60</v>
@@ -5690,7 +5690,7 @@
       </c>
       <c r="K51" s="45"/>
     </row>
-    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="C52" s="29">
         <f>IF(E52&lt;&gt;"",SUBTOTAL(103,E$22:E52),"")</f>
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>44</v>
@@ -5725,7 +5725,7 @@
       </c>
       <c r="K52" s="45"/>
     </row>
-    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5734,7 +5734,7 @@
       </c>
       <c r="C53" s="29">
         <f>IF(E53&lt;&gt;"",SUBTOTAL(103,E$22:E53),"")</f>
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>60</v>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="K53" s="45"/>
     </row>
-    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="C54" s="29">
         <f>IF(E54&lt;&gt;"",SUBTOTAL(103,E$22:E54),"")</f>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>44</v>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="K54" s="45"/>
     </row>
-    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="C55" s="29">
         <f>IF(E55&lt;&gt;"",SUBTOTAL(103,E$22:E55),"")</f>
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="D55" s="30" t="s">
         <v>60</v>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="K55" s="45"/>
     </row>
-    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5839,7 +5839,7 @@
       </c>
       <c r="C56" s="29">
         <f>IF(E56&lt;&gt;"",SUBTOTAL(103,E$22:E56),"")</f>
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>44</v>
@@ -5865,7 +5865,7 @@
       </c>
       <c r="K56" s="45"/>
     </row>
-    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="18" t="s">
         <v>157</v>
       </c>
@@ -5874,7 +5874,7 @@
       </c>
       <c r="C57" s="29">
         <f>IF(E57&lt;&gt;"",SUBTOTAL(103,E$22:E57),"")</f>
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="D57" s="30" t="s">
         <v>60</v>
@@ -5900,7 +5900,7 @@
       </c>
       <c r="K57" s="45"/>
     </row>
-    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5909,7 +5909,7 @@
       </c>
       <c r="C58" s="29">
         <f>IF(E58&lt;&gt;"",SUBTOTAL(103,E$22:E58),"")</f>
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="D58" s="30" t="s">
         <v>44</v>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="K58" s="45"/>
     </row>
-    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="C59" s="29">
         <f>IF(E59&lt;&gt;"",SUBTOTAL(103,E$22:E59),"")</f>
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="D59" s="30" t="s">
         <v>44</v>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="K59" s="45"/>
     </row>
-    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="18" t="s">
         <v>200</v>
       </c>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="C60" s="29">
         <f>IF(E60&lt;&gt;"",SUBTOTAL(103,E$22:E60),"")</f>
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="D60" s="30" t="s">
         <v>60</v>
@@ -6005,12 +6005,12 @@
       </c>
       <c r="K60" s="46"/>
     </row>
-    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61"/>
       <c r="B61"/>
       <c r="C61" s="29">
         <f>IF(E61&lt;&gt;"",SUBTOTAL(103,E$22:E61),"")</f>
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="D61" s="30" t="s">
         <v>44</v>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="K61" s="47"/>
     </row>
-    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="18" t="s">
         <v>138</v>
       </c>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="C62" s="29">
         <f>IF(E62&lt;&gt;"",SUBTOTAL(103,E$22:E62),"")</f>
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="D62" s="30" t="s">
         <v>72</v>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="K62" s="45"/>
     </row>
-    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="C63" s="29">
         <f>IF(E63&lt;&gt;"",SUBTOTAL(103,E$22:E63),"")</f>
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="D63" s="51" t="s">
         <v>72</v>
@@ -6106,7 +6106,7 @@
       </c>
       <c r="K63" s="45"/>
     </row>
-    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6115,7 +6115,7 @@
       </c>
       <c r="C64" s="29">
         <f>IF(E64&lt;&gt;"",SUBTOTAL(103,E$22:E64),"")</f>
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="D64" s="30" t="s">
         <v>60</v>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="K64" s="45"/>
     </row>
-    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="18" t="s">
         <v>145</v>
       </c>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="C65" s="29">
         <f>IF(E65&lt;&gt;"",SUBTOTAL(103,E$22:E65),"")</f>
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="D65" s="30" t="s">
         <v>44</v>
@@ -6176,7 +6176,7 @@
       </c>
       <c r="K65" s="45"/>
     </row>
-    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6185,7 +6185,7 @@
       </c>
       <c r="C66" s="29">
         <f>IF(E66&lt;&gt;"",SUBTOTAL(103,E$22:E66),"")</f>
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="D66" s="30" t="s">
         <v>44</v>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="K66" s="44"/>
     </row>
-    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="C67" s="29">
         <f>IF(E67&lt;&gt;"",SUBTOTAL(103,E$22:E67),"")</f>
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="D67" s="30" t="s">
         <v>44</v>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="K67" s="45"/>
     </row>
-    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="18" t="s">
         <v>151</v>
       </c>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="C68" s="29">
         <f>IF(E68&lt;&gt;"",SUBTOTAL(103,E$22:E68),"")</f>
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="D68" s="30" t="s">
         <v>44</v>
@@ -6281,7 +6281,7 @@
       </c>
       <c r="K68" s="45"/>
     </row>
-    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6290,7 +6290,7 @@
       </c>
       <c r="C69" s="29">
         <f>IF(E69&lt;&gt;"",SUBTOTAL(103,E$22:E69),"")</f>
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="D69" s="30" t="s">
         <v>44</v>
@@ -6316,7 +6316,7 @@
       </c>
       <c r="K69" s="45"/>
     </row>
-    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="18" t="s">
         <v>56</v>
       </c>
@@ -6325,7 +6325,7 @@
       </c>
       <c r="C70" s="29">
         <f>IF(E70&lt;&gt;"",SUBTOTAL(103,E$22:E70),"")</f>
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="D70" s="30" t="s">
         <v>44</v>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="K70" s="45"/>
     </row>
-    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="18" t="s">
         <v>63</v>
       </c>
@@ -6360,7 +6360,7 @@
       </c>
       <c r="C71" s="29">
         <f>IF(E71&lt;&gt;"",SUBTOTAL(103,E$22:E71),"")</f>
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="D71" s="30" t="s">
         <v>44</v>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="K71" s="45"/>
     </row>
-    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="18" t="s">
         <v>65</v>
       </c>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="C72" s="29">
         <f>IF(E72&lt;&gt;"",SUBTOTAL(103,E$22:E72),"")</f>
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="D72" s="30" t="s">
         <v>44</v>
@@ -6421,7 +6421,7 @@
       </c>
       <c r="K72" s="45"/>
     </row>
-    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="C73" s="29">
         <f>IF(E73&lt;&gt;"",SUBTOTAL(103,E$22:E73),"")</f>
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="D73" s="30" t="s">
         <v>44</v>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="K73" s="45"/>
     </row>
-    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="C74" s="29">
         <f>IF(E74&lt;&gt;"",SUBTOTAL(103,E$22:E74),"")</f>
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>44</v>
@@ -6491,7 +6491,7 @@
       </c>
       <c r="K74" s="45"/>
     </row>
-    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6500,7 +6500,7 @@
       </c>
       <c r="C75" s="29">
         <f>IF(E75&lt;&gt;"",SUBTOTAL(103,E$22:E75),"")</f>
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="D75" s="30" t="s">
         <v>44</v>
@@ -6526,7 +6526,7 @@
       </c>
       <c r="K75" s="45"/>
     </row>
-    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="18" t="s">
         <v>167</v>
       </c>
@@ -6535,7 +6535,7 @@
       </c>
       <c r="C76" s="29">
         <f>IF(E76&lt;&gt;"",SUBTOTAL(103,E$22:E76),"")</f>
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="D76" s="30" t="s">
         <v>44</v>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="K76" s="45"/>
     </row>
-    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6570,7 +6570,7 @@
       </c>
       <c r="C77" s="29">
         <f>IF(E77&lt;&gt;"",SUBTOTAL(103,E$22:E77),"")</f>
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="D77" s="30" t="s">
         <v>44</v>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="K77" s="45"/>
     </row>
-    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="18" t="s">
         <v>105</v>
       </c>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="C78" s="29">
         <f>IF(E78&lt;&gt;"",SUBTOTAL(103,E$22:E78),"")</f>
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="D78" s="30" t="s">
         <v>44</v>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="K78" s="45"/>
     </row>
-    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="18" t="s">
         <v>173</v>
       </c>
@@ -6640,7 +6640,7 @@
       </c>
       <c r="C79" s="29">
         <f>IF(E79&lt;&gt;"",SUBTOTAL(103,E$22:E79),"")</f>
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="D79" s="30" t="s">
         <v>60</v>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="K79" s="45"/>
     </row>
-    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="C80" s="29">
         <f>IF(E80&lt;&gt;"",SUBTOTAL(103,E$22:E80),"")</f>
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="D80" s="30" t="s">
         <v>44</v>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="K80" s="45"/>
     </row>
-    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6710,7 +6710,7 @@
       </c>
       <c r="C81" s="29">
         <f>IF(E81&lt;&gt;"",SUBTOTAL(103,E$22:E81),"")</f>
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="D81" s="30" t="s">
         <v>72</v>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="K81" s="45"/>
     </row>
-    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6745,7 +6745,7 @@
       </c>
       <c r="C82" s="29">
         <f>IF(E82&lt;&gt;"",SUBTOTAL(103,E$22:E82),"")</f>
-        <v>61</v>
+        <v>1</v>
       </c>
       <c r="D82" s="30" t="s">
         <v>44</v>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="K82" s="45"/>
     </row>
-    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="C83" s="29">
         <f>IF(E83&lt;&gt;"",SUBTOTAL(103,E$22:E83),"")</f>
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="D83" s="30" t="s">
         <v>44</v>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="K83" s="45"/>
     </row>
-    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6815,7 +6815,7 @@
       </c>
       <c r="C84" s="29">
         <f>IF(E84&lt;&gt;"",SUBTOTAL(103,E$22:E84),"")</f>
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D84" s="30" t="s">
         <v>72</v>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="K84" s="45"/>
     </row>
-    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" s="36" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6850,7 +6850,7 @@
       </c>
       <c r="C85" s="29">
         <f>IF(E85&lt;&gt;"",SUBTOTAL(103,E$22:E85),"")</f>
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="D85" s="30" t="s">
         <v>72</v>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="K85" s="45"/>
     </row>
-    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="C86" s="29">
         <f>IF(E86&lt;&gt;"",SUBTOTAL(103,E$22:E86),"")</f>
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="D86" s="30" t="s">
         <v>60</v>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="K86" s="45"/>
     </row>
-    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" s="36" customFormat="1" ht="30.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6920,7 +6920,7 @@
       </c>
       <c r="C87" s="29">
         <f>IF(E87&lt;&gt;"",SUBTOTAL(103,E$22:E87),"")</f>
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="D87" s="30" t="s">
         <v>72</v>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="K87" s="45"/>
     </row>
-    <row r="88" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="18" t="s">
         <v>194</v>
       </c>
@@ -6955,7 +6955,7 @@
       </c>
       <c r="C88" s="29">
         <f>IF(E88&lt;&gt;"",SUBTOTAL(103,E$22:E88),"")</f>
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="D88" s="30" t="s">
         <v>44</v>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="K88" s="46"/>
     </row>
-    <row r="89" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="C89" s="29">
         <f>IF(E89&lt;&gt;"",SUBTOTAL(103,E$22:E89),"")</f>
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="D89" s="30" t="s">
         <v>44</v>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="K89" s="46"/>
     </row>
-    <row r="90" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7025,7 +7025,7 @@
       </c>
       <c r="C90" s="29">
         <f>IF(E90&lt;&gt;"",SUBTOTAL(103,E$22:E90),"")</f>
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="D90" s="30" t="s">
         <v>44</v>
@@ -7051,7 +7051,7 @@
       </c>
       <c r="K90" s="46"/>
     </row>
-    <row r="91" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" ht="27.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7060,7 +7060,7 @@
       </c>
       <c r="C91" s="29">
         <f>IF(E91&lt;&gt;"",SUBTOTAL(103,E$22:E91),"")</f>
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="D91" s="30" t="s">
         <v>44</v>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="K91" s="45"/>
     </row>
-    <row r="92" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="C92" s="29">
         <f>IF(E92&lt;&gt;"",SUBTOTAL(103,E$22:E92),"")</f>
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="D92" s="30" t="s">
         <v>60</v>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="K92" s="46"/>
     </row>
-    <row r="93" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="18" t="s">
         <v>204</v>
       </c>
@@ -7130,7 +7130,7 @@
       </c>
       <c r="C93" s="29">
         <f>IF(E93&lt;&gt;"",SUBTOTAL(103,E$22:E93),"")</f>
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="D93" s="30" t="s">
         <v>60</v>
@@ -7156,7 +7156,7 @@
       </c>
       <c r="K93" s="46"/>
     </row>
-    <row r="94" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7165,7 +7165,7 @@
       </c>
       <c r="C94" s="29">
         <f>IF(E94&lt;&gt;"",SUBTOTAL(103,E$22:E94),"")</f>
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="D94" s="30" t="s">
         <v>44</v>
@@ -7191,7 +7191,7 @@
       </c>
       <c r="K94" s="46"/>
     </row>
-    <row r="95" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="C95" s="29">
         <f>IF(E95&lt;&gt;"",SUBTOTAL(103,E$22:E95),"")</f>
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="D95" s="30" t="s">
         <v>44</v>
@@ -7226,10 +7226,10 @@
       </c>
       <c r="K95" s="46"/>
     </row>
-    <row r="96" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C96" s="29">
         <f>IF(E96&lt;&gt;"",SUBTOTAL(103,E$22:E96),"")</f>
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="D96" s="30" t="s">
         <v>44</v>
@@ -7255,10 +7255,10 @@
       </c>
       <c r="K96" s="46"/>
     </row>
-    <row r="97" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C97" s="29">
         <f>IF(E97&lt;&gt;"",SUBTOTAL(103,E$22:E97),"")</f>
-        <v>76</v>
+        <v>1</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>44</v>
@@ -7284,10 +7284,10 @@
       </c>
       <c r="K97" s="46"/>
     </row>
-    <row r="98" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C98" s="29">
         <f>IF(E98&lt;&gt;"",SUBTOTAL(103,E$22:E98),"")</f>
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>44</v>
@@ -7313,10 +7313,10 @@
       </c>
       <c r="K98" s="46"/>
     </row>
-    <row r="99" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C99" s="29">
         <f>IF(E99&lt;&gt;"",SUBTOTAL(103,E$22:E99),"")</f>
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="D99" s="30" t="s">
         <v>60</v>
@@ -7342,10 +7342,10 @@
       </c>
       <c r="K99" s="46"/>
     </row>
-    <row r="100" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C100" s="29">
         <f>IF(E100&lt;&gt;"",SUBTOTAL(103,E$22:E100),"")</f>
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="D100" s="30" t="s">
         <v>60</v>
@@ -7373,10 +7373,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="101" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C101" s="29">
         <f>IF(E101&lt;&gt;"",SUBTOTAL(103,E$22:E101),"")</f>
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="D101" s="30" t="s">
         <v>72</v>
@@ -7402,7 +7402,7 @@
       </c>
       <c r="K101" s="47"/>
     </row>
-    <row r="102" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="18" t="e">
         <v>#N/A</v>
       </c>
@@ -7411,7 +7411,7 @@
       </c>
       <c r="C102" s="29">
         <f>IF(E102&lt;&gt;"",SUBTOTAL(103,E$22:E102),"")</f>
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="D102" s="30" t="s">
         <v>44</v>
@@ -7437,10 +7437,10 @@
       </c>
       <c r="K102" s="45"/>
     </row>
-    <row r="103" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C103" s="29">
         <f>IF(E103&lt;&gt;"",SUBTOTAL(103,E$22:E103),"")</f>
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="D103" s="30" t="s">
         <v>44</v>
@@ -7466,10 +7466,10 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C104" s="29">
         <f>IF(E104&lt;&gt;"",SUBTOTAL(103,E$22:E104),"")</f>
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="D104" s="30" t="s">
         <v>60</v>
@@ -7495,10 +7495,10 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C105" s="29">
         <f>IF(E105&lt;&gt;"",SUBTOTAL(103,E$22:E105),"")</f>
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="D105" s="30" t="s">
         <v>60</v>
@@ -7524,10 +7524,10 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C106" s="29">
         <f>IF(E106&lt;&gt;"",SUBTOTAL(103,E$22:E106),"")</f>
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="D106" s="30" t="s">
         <v>44</v>
@@ -7553,10 +7553,10 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C107" s="29">
         <f>IF(E107&lt;&gt;"",SUBTOTAL(103,E$22:E107),"")</f>
-        <v>86</v>
+        <v>1</v>
       </c>
       <c r="D107" s="30" t="s">
         <v>44</v>
@@ -7582,10 +7582,10 @@
       </c>
       <c r="K107" s="47"/>
     </row>
-    <row r="108" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C108" s="29">
         <f>IF(E108&lt;&gt;"",SUBTOTAL(103,E$22:E108),"")</f>
-        <v>87</v>
+        <v>1</v>
       </c>
       <c r="D108" s="30" t="s">
         <v>44</v>
@@ -7611,10 +7611,10 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C109" s="29">
         <f>IF(E109&lt;&gt;"",SUBTOTAL(103,E$22:E109),"")</f>
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="D109" s="30" t="s">
         <v>44</v>
@@ -7640,10 +7640,10 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C110" s="29">
         <f>IF(E110&lt;&gt;"",SUBTOTAL(103,E$22:E110),"")</f>
-        <v>89</v>
+        <v>1</v>
       </c>
       <c r="D110" s="30" t="s">
         <v>60</v>
@@ -7669,10 +7669,10 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C111" s="29">
         <f>IF(E111&lt;&gt;"",SUBTOTAL(103,E$22:E111),"")</f>
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="D111" s="30" t="s">
         <v>60</v>
@@ -7701,7 +7701,7 @@
     <row r="112" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C112" s="29">
         <f>IF(E112&lt;&gt;"",SUBTOTAL(103,E$22:E112),"")</f>
-        <v>91</v>
+        <v>2</v>
       </c>
       <c r="D112" s="30" t="s">
         <v>44</v>
@@ -7727,10 +7727,10 @@
       </c>
       <c r="K112" s="47"/>
     </row>
-    <row r="113" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C113" s="29">
         <f>IF(E113&lt;&gt;"",SUBTOTAL(103,E$22:E113),"")</f>
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="D113" s="30" t="s">
         <v>60</v>
@@ -7756,10 +7756,10 @@
       </c>
       <c r="K113" s="47"/>
     </row>
-    <row r="114" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C114" s="29">
         <f>IF(E114&lt;&gt;"",SUBTOTAL(103,E$22:E114),"")</f>
-        <v>93</v>
+        <v>2</v>
       </c>
       <c r="D114" s="30" t="s">
         <v>60</v>
@@ -7785,10 +7785,10 @@
       </c>
       <c r="K114" s="47"/>
     </row>
-    <row r="115" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C115" s="29">
         <f>IF(E115&lt;&gt;"",SUBTOTAL(103,E$22:E115),"")</f>
-        <v>94</v>
+        <v>2</v>
       </c>
       <c r="D115" s="30" t="s">
         <v>60</v>
@@ -7814,10 +7814,10 @@
       </c>
       <c r="K115" s="47"/>
     </row>
-    <row r="116" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C116" s="29">
         <f>IF(E116&lt;&gt;"",SUBTOTAL(103,E$22:E116),"")</f>
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="D116" s="30" t="s">
         <v>60</v>
@@ -7843,10 +7843,10 @@
       </c>
       <c r="K116" s="47"/>
     </row>
-    <row r="117" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C117" s="29">
         <f>IF(E117&lt;&gt;"",SUBTOTAL(103,E$22:E117),"")</f>
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="D117" s="30" t="s">
         <v>72</v>
@@ -7872,10 +7872,10 @@
       </c>
       <c r="K117" s="47"/>
     </row>
-    <row r="118" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C118" s="29">
         <f>IF(E118&lt;&gt;"",SUBTOTAL(103,E$22:E118),"")</f>
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="D118" s="30" t="s">
         <v>44</v>
@@ -7901,7 +7901,7 @@
       </c>
       <c r="K118" s="47"/>
     </row>
-    <row r="119" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="18" t="s">
         <v>163</v>
       </c>
@@ -7910,7 +7910,7 @@
       </c>
       <c r="C119" s="29">
         <f>IF(E119&lt;&gt;"",SUBTOTAL(103,E$22:E119),"")</f>
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="D119" s="30" t="s">
         <v>44</v>
@@ -7936,10 +7936,10 @@
       </c>
       <c r="K119" s="45"/>
     </row>
-    <row r="120" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C120" s="29">
         <f>IF(E120&lt;&gt;"",SUBTOTAL(103,E$22:E120),"")</f>
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="D120" s="30" t="s">
         <v>44</v>
@@ -7965,10 +7965,10 @@
       </c>
       <c r="K120" s="47"/>
     </row>
-    <row r="121" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C121" s="29">
         <f>IF(E121&lt;&gt;"",SUBTOTAL(103,E$22:E121),"")</f>
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="D121" s="30" t="s">
         <v>72</v>
@@ -7993,10 +7993,10 @@
       </c>
       <c r="K121" s="47"/>
     </row>
-    <row r="122" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C122" s="29">
         <f>IF(E122&lt;&gt;"",SUBTOTAL(103,E$22:E122),"")</f>
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="D122" s="30" t="s">
         <v>44</v>
@@ -8021,10 +8021,10 @@
       </c>
       <c r="K122" s="47"/>
     </row>
-    <row r="123" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C123" s="29">
         <f>IF(E123&lt;&gt;"",SUBTOTAL(103,E$22:E123),"")</f>
-        <v>102</v>
+        <v>2</v>
       </c>
       <c r="D123" s="30" t="s">
         <v>60</v>
@@ -8049,10 +8049,10 @@
       </c>
       <c r="K123" s="47"/>
     </row>
-    <row r="124" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C124" s="29">
         <f>IF(E124&lt;&gt;"",SUBTOTAL(103,E$22:E124),"")</f>
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="D124" s="30" t="s">
         <v>60</v>
@@ -8077,10 +8077,10 @@
       </c>
       <c r="K124" s="47"/>
     </row>
-    <row r="125" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C125" s="29">
         <f>IF(E125&lt;&gt;"",SUBTOTAL(103,E$22:E125),"")</f>
-        <v>104</v>
+        <v>2</v>
       </c>
       <c r="D125" s="30" t="s">
         <v>44</v>
@@ -8105,10 +8105,10 @@
       </c>
       <c r="K125" s="47"/>
     </row>
-    <row r="126" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C126" s="29">
         <f>IF(E126&lt;&gt;"",SUBTOTAL(103,E$22:E126),"")</f>
-        <v>105</v>
+        <v>2</v>
       </c>
       <c r="D126" s="30" t="s">
         <v>60</v>
@@ -8133,10 +8133,10 @@
       </c>
       <c r="K126" s="47"/>
     </row>
-    <row r="127" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C127" s="29">
         <f>IF(E127&lt;&gt;"",SUBTOTAL(103,E$22:E127),"")</f>
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="D127" s="30" t="s">
         <v>60</v>
@@ -8161,10 +8161,10 @@
       </c>
       <c r="K127" s="47"/>
     </row>
-    <row r="128" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C128" s="29">
         <f>IF(E128&lt;&gt;"",SUBTOTAL(103,E$22:E128),"")</f>
-        <v>107</v>
+        <v>2</v>
       </c>
       <c r="D128" s="30" t="s">
         <v>44</v>
@@ -8189,10 +8189,10 @@
       </c>
       <c r="K128" s="47"/>
     </row>
-    <row r="129" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C129" s="29">
         <f>IF(E129&lt;&gt;"",SUBTOTAL(103,E$22:E129),"")</f>
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="D129" s="30" t="s">
         <v>44</v>
@@ -8217,10 +8217,10 @@
       </c>
       <c r="K129" s="47"/>
     </row>
-    <row r="130" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C130" s="42">
         <f>IF(E130&lt;&gt;"",SUBTOTAL(103,E$22:E130),"")</f>
-        <v>109</v>
+        <v>2</v>
       </c>
       <c r="D130" s="30" t="s">
         <v>44</v>
@@ -8245,10 +8245,10 @@
       </c>
       <c r="K130" s="47"/>
     </row>
-    <row r="131" spans="3:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:11" ht="29.25" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C131" s="42">
         <f>IF(E131&lt;&gt;"",SUBTOTAL(103,E$22:E131),"")</f>
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="D131" s="30" t="s">
         <v>44</v>
@@ -8273,10 +8273,10 @@
       </c>
       <c r="K131" s="47"/>
     </row>
-    <row r="132" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C132" s="42">
         <f>IF(E132&lt;&gt;"",SUBTOTAL(103,E$22:E132),"")</f>
-        <v>111</v>
+        <v>2</v>
       </c>
       <c r="D132" s="30" t="s">
         <v>60</v>
@@ -8301,10 +8301,10 @@
       </c>
       <c r="K132" s="47"/>
     </row>
-    <row r="133" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C133" s="42">
         <f>IF(E133&lt;&gt;"",SUBTOTAL(103,E$22:E133),"")</f>
-        <v>112</v>
+        <v>2</v>
       </c>
       <c r="D133" s="30" t="s">
         <v>44</v>
@@ -8329,10 +8329,10 @@
       </c>
       <c r="K133" s="47"/>
     </row>
-    <row r="134" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C134" s="42">
         <f>IF(E134&lt;&gt;"",SUBTOTAL(103,E$22:E134),"")</f>
-        <v>113</v>
+        <v>2</v>
       </c>
       <c r="D134" s="30" t="s">
         <v>44</v>
@@ -8359,10 +8359,10 @@
         <v>315</v>
       </c>
     </row>
-    <row r="135" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C135" s="42">
         <f>IF(E135&lt;&gt;"",SUBTOTAL(103,E$22:E135),"")</f>
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="D135" s="30" t="s">
         <v>72</v>
@@ -8387,10 +8387,10 @@
       </c>
       <c r="K135" s="46"/>
     </row>
-    <row r="136" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C136" s="42">
         <f>IF(E136&lt;&gt;"",SUBTOTAL(103,E$22:E136),"")</f>
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="D136" s="30" t="s">
         <v>60</v>
@@ -8415,10 +8415,10 @@
       </c>
       <c r="K136" s="46"/>
     </row>
-    <row r="137" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C137" s="42">
         <f>IF(E137&lt;&gt;"",SUBTOTAL(103,E$22:E137),"")</f>
-        <v>116</v>
+        <v>2</v>
       </c>
       <c r="D137" s="30" t="s">
         <v>44</v>
@@ -8443,10 +8443,10 @@
       </c>
       <c r="K137" s="46"/>
     </row>
-    <row r="138" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C138" s="42">
         <f>IF(E138&lt;&gt;"",SUBTOTAL(103,E$22:E138),"")</f>
-        <v>117</v>
+        <v>2</v>
       </c>
       <c r="D138" s="30" t="s">
         <v>60</v>
@@ -8471,10 +8471,10 @@
       </c>
       <c r="K138" s="46"/>
     </row>
-    <row r="139" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C139" s="42">
         <f>IF(E139&lt;&gt;"",SUBTOTAL(103,E$22:E139),"")</f>
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="D139" s="30" t="s">
         <v>44</v>
@@ -8499,10 +8499,10 @@
       </c>
       <c r="K139" s="46"/>
     </row>
-    <row r="140" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C140" s="42">
         <f>IF(E140&lt;&gt;"",SUBTOTAL(103,E$22:E140),"")</f>
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="D140" s="30" t="s">
         <v>44</v>
@@ -8530,10 +8530,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="141" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C141" s="42">
         <f>IF(E141&lt;&gt;"",SUBTOTAL(103,E$22:E141),"")</f>
-        <v>120</v>
+        <v>2</v>
       </c>
       <c r="D141" s="30" t="s">
         <v>44</v>
@@ -8561,10 +8561,10 @@
         <v>310</v>
       </c>
     </row>
-    <row r="142" spans="3:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="3:11" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="42">
         <f>IF(E142&lt;&gt;"",SUBTOTAL(103,E$22:E142),"")</f>
-        <v>121</v>
+        <v>2</v>
       </c>
       <c r="D142" s="30" t="s">
         <v>72</v>
@@ -8620,7 +8620,14 @@
       <c r="K143" s="47"/>
     </row>
   </sheetData>
-  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}"/>
+  <autoFilter ref="A21:K142" xr:uid="{C3D77B87-320E-4CAC-BE20-C9B51A590042}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="Danh Tiền"/>
+        <filter val="Lê Cao Tài"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>